<commit_message>
Actualizacion dashboard por agente
</commit_message>
<xml_diff>
--- a/public/Week 10.8.xlsx
+++ b/public/Week 10.8.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$T$662</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -6302,7 +6305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:T662"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
   <sheetData>
@@ -6368,7 +6371,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" ht="23" customHeight="1" spans="1:20">
+    <row r="2" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
@@ -6460,7 +6463,7 @@
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
     </row>
-    <row r="4" ht="23" customHeight="1" spans="1:20">
+    <row r="4" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A4" s="2" t="s">
         <v>37</v>
       </c>
@@ -6506,7 +6509,7 @@
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
     </row>
-    <row r="5" ht="23" customHeight="1" spans="1:20">
+    <row r="5" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A5" s="2" t="s">
         <v>42</v>
       </c>
@@ -6552,7 +6555,7 @@
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
     </row>
-    <row r="6" ht="23" customHeight="1" spans="1:20">
+    <row r="6" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A6" s="2" t="s">
         <v>46</v>
       </c>
@@ -6598,7 +6601,7 @@
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
     </row>
-    <row r="7" ht="23" customHeight="1" spans="1:20">
+    <row r="7" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A7" s="2" t="s">
         <v>49</v>
       </c>
@@ -6644,7 +6647,7 @@
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
     </row>
-    <row r="8" ht="23" customHeight="1" spans="1:20">
+    <row r="8" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A8" s="2" t="s">
         <v>54</v>
       </c>
@@ -6736,7 +6739,7 @@
       <c r="S9" s="2"/>
       <c r="T9" s="2"/>
     </row>
-    <row r="10" ht="23" customHeight="1" spans="1:20">
+    <row r="10" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A10" s="2" t="s">
         <v>60</v>
       </c>
@@ -6790,7 +6793,7 @@
       </c>
       <c r="T10" s="2"/>
     </row>
-    <row r="11" ht="23" customHeight="1" spans="1:20">
+    <row r="11" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A11" s="2" t="s">
         <v>66</v>
       </c>
@@ -6836,7 +6839,7 @@
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
     </row>
-    <row r="12" ht="23" customHeight="1" spans="1:20">
+    <row r="12" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A12" s="2" t="s">
         <v>71</v>
       </c>
@@ -6882,7 +6885,7 @@
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
     </row>
-    <row r="13" ht="23" customHeight="1" spans="1:20">
+    <row r="13" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A13" s="2" t="s">
         <v>74</v>
       </c>
@@ -6928,7 +6931,7 @@
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
     </row>
-    <row r="14" ht="23" customHeight="1" spans="1:20">
+    <row r="14" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A14" s="2" t="s">
         <v>77</v>
       </c>
@@ -7028,7 +7031,7 @@
       <c r="S15" s="2"/>
       <c r="T15" s="2"/>
     </row>
-    <row r="16" ht="23" customHeight="1" spans="1:20">
+    <row r="16" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A16" s="2" t="s">
         <v>84</v>
       </c>
@@ -7078,7 +7081,7 @@
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
     </row>
-    <row r="17" ht="23" customHeight="1" spans="1:20">
+    <row r="17" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A17" s="2" t="s">
         <v>89</v>
       </c>
@@ -7124,7 +7127,7 @@
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
     </row>
-    <row r="18" ht="23" customHeight="1" spans="1:20">
+    <row r="18" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A18" s="2" t="s">
         <v>92</v>
       </c>
@@ -7170,7 +7173,7 @@
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
     </row>
-    <row r="19" ht="23" customHeight="1" spans="1:20">
+    <row r="19" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A19" s="2" t="s">
         <v>95</v>
       </c>
@@ -7216,7 +7219,7 @@
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
     </row>
-    <row r="20" ht="23" customHeight="1" spans="1:20">
+    <row r="20" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A20" s="2" t="s">
         <v>98</v>
       </c>
@@ -7316,7 +7319,7 @@
       <c r="S21" s="2"/>
       <c r="T21" s="2"/>
     </row>
-    <row r="22" ht="23" customHeight="1" spans="1:20">
+    <row r="22" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A22" s="2" t="s">
         <v>106</v>
       </c>
@@ -7362,7 +7365,7 @@
       <c r="S22" s="2"/>
       <c r="T22" s="2"/>
     </row>
-    <row r="23" ht="23" customHeight="1" spans="1:20">
+    <row r="23" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A23" s="2" t="s">
         <v>110</v>
       </c>
@@ -7408,7 +7411,7 @@
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
     </row>
-    <row r="24" ht="23" customHeight="1" spans="1:20">
+    <row r="24" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A24" s="2" t="s">
         <v>113</v>
       </c>
@@ -7454,7 +7457,7 @@
       <c r="S24" s="2"/>
       <c r="T24" s="2"/>
     </row>
-    <row r="25" ht="23" customHeight="1" spans="1:20">
+    <row r="25" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A25" s="2" t="s">
         <v>117</v>
       </c>
@@ -7508,7 +7511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" ht="23" customHeight="1" spans="1:20">
+    <row r="26" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A26" s="2" t="s">
         <v>121</v>
       </c>
@@ -7618,7 +7621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" ht="23" customHeight="1" spans="1:20">
+    <row r="28" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A28" s="2" t="s">
         <v>128</v>
       </c>
@@ -7668,7 +7671,7 @@
       <c r="S28" s="2"/>
       <c r="T28" s="2"/>
     </row>
-    <row r="29" ht="23" customHeight="1" spans="1:20">
+    <row r="29" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A29" s="2" t="s">
         <v>132</v>
       </c>
@@ -7718,7 +7721,7 @@
       <c r="S29" s="2"/>
       <c r="T29" s="2"/>
     </row>
-    <row r="30" ht="23" customHeight="1" spans="1:20">
+    <row r="30" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A30" s="2" t="s">
         <v>135</v>
       </c>
@@ -7774,7 +7777,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" ht="23" customHeight="1" spans="1:20">
+    <row r="31" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A31" s="2" t="s">
         <v>138</v>
       </c>
@@ -7826,7 +7829,7 @@
       <c r="S31" s="2"/>
       <c r="T31" s="2"/>
     </row>
-    <row r="32" ht="23" customHeight="1" spans="1:20">
+    <row r="32" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A32" s="2" t="s">
         <v>143</v>
       </c>
@@ -7934,7 +7937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" ht="23" customHeight="1" spans="1:20">
+    <row r="34" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A34" s="2" t="s">
         <v>147</v>
       </c>
@@ -7988,7 +7991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" ht="23" customHeight="1" spans="1:20">
+    <row r="35" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A35" s="2" t="s">
         <v>150</v>
       </c>
@@ -8044,7 +8047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" ht="23" customHeight="1" spans="1:20">
+    <row r="36" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A36" s="2" t="s">
         <v>154</v>
       </c>
@@ -8098,7 +8101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" ht="23" customHeight="1" spans="1:20">
+    <row r="37" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A37" s="2" t="s">
         <v>157</v>
       </c>
@@ -8148,7 +8151,7 @@
       <c r="S37" s="2"/>
       <c r="T37" s="2"/>
     </row>
-    <row r="38" ht="23" customHeight="1" spans="1:20">
+    <row r="38" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A38" s="2" t="s">
         <v>161</v>
       </c>
@@ -8258,7 +8261,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" ht="23" customHeight="1" spans="1:20">
+    <row r="40" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A40" s="2" t="s">
         <v>167</v>
       </c>
@@ -8308,7 +8311,7 @@
       <c r="S40" s="2"/>
       <c r="T40" s="2"/>
     </row>
-    <row r="41" ht="23" customHeight="1" spans="1:20">
+    <row r="41" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A41" s="2" t="s">
         <v>170</v>
       </c>
@@ -8358,7 +8361,7 @@
       <c r="S41" s="2"/>
       <c r="T41" s="2"/>
     </row>
-    <row r="42" ht="23" customHeight="1" spans="1:20">
+    <row r="42" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A42" s="2" t="s">
         <v>172</v>
       </c>
@@ -8412,7 +8415,7 @@
       </c>
       <c r="T42" s="2"/>
     </row>
-    <row r="43" ht="23" customHeight="1" spans="1:20">
+    <row r="43" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A43" s="2" t="s">
         <v>176</v>
       </c>
@@ -8466,7 +8469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" ht="23" customHeight="1" spans="1:20">
+    <row r="44" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A44" s="2" t="s">
         <v>178</v>
       </c>
@@ -8574,7 +8577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" ht="23" customHeight="1" spans="1:20">
+    <row r="46" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A46" s="2" t="s">
         <v>187</v>
       </c>
@@ -8630,7 +8633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" ht="23" customHeight="1" spans="1:20">
+    <row r="47" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A47" s="2" t="s">
         <v>189</v>
       </c>
@@ -8684,7 +8687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" ht="23" customHeight="1" spans="1:20">
+    <row r="48" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A48" s="2" t="s">
         <v>192</v>
       </c>
@@ -8738,7 +8741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" ht="23" customHeight="1" spans="1:20">
+    <row r="49" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A49" s="2" t="s">
         <v>194</v>
       </c>
@@ -8794,7 +8797,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" ht="23" customHeight="1" spans="1:20">
+    <row r="50" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A50" s="2" t="s">
         <v>198</v>
       </c>
@@ -8898,7 +8901,7 @@
       <c r="S51" s="2"/>
       <c r="T51" s="2"/>
     </row>
-    <row r="52" ht="23" customHeight="1" spans="1:20">
+    <row r="52" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A52" s="2" t="s">
         <v>204</v>
       </c>
@@ -8954,7 +8957,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" ht="23" customHeight="1" spans="1:20">
+    <row r="53" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A53" s="2" t="s">
         <v>207</v>
       </c>
@@ -9006,7 +9009,7 @@
       <c r="S53" s="2"/>
       <c r="T53" s="2"/>
     </row>
-    <row r="54" ht="23" customHeight="1" spans="1:20">
+    <row r="54" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A54" s="2" t="s">
         <v>211</v>
       </c>
@@ -9060,7 +9063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" ht="23" customHeight="1" spans="1:20">
+    <row r="55" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A55" s="2" t="s">
         <v>214</v>
       </c>
@@ -9114,7 +9117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" ht="23" customHeight="1" spans="1:20">
+    <row r="56" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A56" s="2" t="s">
         <v>217</v>
       </c>
@@ -9214,7 +9217,7 @@
       <c r="S57" s="2"/>
       <c r="T57" s="2"/>
     </row>
-    <row r="58" ht="23" customHeight="1" spans="1:20">
+    <row r="58" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A58" s="2" t="s">
         <v>226</v>
       </c>
@@ -9266,7 +9269,7 @@
       <c r="S58" s="2"/>
       <c r="T58" s="2"/>
     </row>
-    <row r="59" ht="23" customHeight="1" spans="1:20">
+    <row r="59" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A59" s="2" t="s">
         <v>231</v>
       </c>
@@ -9316,7 +9319,7 @@
       <c r="S59" s="2"/>
       <c r="T59" s="2"/>
     </row>
-    <row r="60" ht="23" customHeight="1" spans="1:20">
+    <row r="60" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A60" s="2" t="s">
         <v>235</v>
       </c>
@@ -9370,7 +9373,7 @@
       </c>
       <c r="T60" s="2"/>
     </row>
-    <row r="61" ht="23" customHeight="1" spans="1:20">
+    <row r="61" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A61" s="2" t="s">
         <v>238</v>
       </c>
@@ -9424,7 +9427,7 @@
       </c>
       <c r="T61" s="2"/>
     </row>
-    <row r="62" ht="23" customHeight="1" spans="1:20">
+    <row r="62" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A62" s="2" t="s">
         <v>242</v>
       </c>
@@ -9526,7 +9529,7 @@
       <c r="S63" s="2"/>
       <c r="T63" s="2"/>
     </row>
-    <row r="64" ht="23" customHeight="1" spans="1:20">
+    <row r="64" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A64" s="2" t="s">
         <v>248</v>
       </c>
@@ -9576,7 +9579,7 @@
       <c r="S64" s="2"/>
       <c r="T64" s="2"/>
     </row>
-    <row r="65" ht="23" customHeight="1" spans="1:20">
+    <row r="65" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A65" s="2" t="s">
         <v>252</v>
       </c>
@@ -9632,7 +9635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" ht="23" customHeight="1" spans="1:20">
+    <row r="66" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A66" s="2" t="s">
         <v>255</v>
       </c>
@@ -9688,7 +9691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" ht="23" customHeight="1" spans="1:20">
+    <row r="67" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A67" s="2" t="s">
         <v>257</v>
       </c>
@@ -9742,7 +9745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" ht="23" customHeight="1" spans="1:20">
+    <row r="68" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A68" s="2" t="s">
         <v>260</v>
       </c>
@@ -9852,7 +9855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" ht="23" customHeight="1" spans="1:20">
+    <row r="70" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A70" s="2" t="s">
         <v>265</v>
       </c>
@@ -9906,7 +9909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" ht="23" customHeight="1" spans="1:20">
+    <row r="71" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A71" s="2" t="s">
         <v>269</v>
       </c>
@@ -9958,7 +9961,7 @@
       <c r="S71" s="2"/>
       <c r="T71" s="2"/>
     </row>
-    <row r="72" ht="23" customHeight="1" spans="1:20">
+    <row r="72" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A72" s="2" t="s">
         <v>274</v>
       </c>
@@ -10008,7 +10011,7 @@
       <c r="S72" s="2"/>
       <c r="T72" s="2"/>
     </row>
-    <row r="73" ht="23" customHeight="1" spans="1:20">
+    <row r="73" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A73" s="2" t="s">
         <v>278</v>
       </c>
@@ -10060,7 +10063,7 @@
       <c r="S73" s="2"/>
       <c r="T73" s="2"/>
     </row>
-    <row r="74" ht="23" customHeight="1" spans="1:20">
+    <row r="74" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A74" s="2" t="s">
         <v>282</v>
       </c>
@@ -10168,7 +10171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" ht="23" customHeight="1" spans="1:20">
+    <row r="76" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A76" s="2" t="s">
         <v>289</v>
       </c>
@@ -10222,7 +10225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" ht="23" customHeight="1" spans="1:20">
+    <row r="77" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A77" s="2" t="s">
         <v>293</v>
       </c>
@@ -10272,7 +10275,7 @@
       <c r="S77" s="2"/>
       <c r="T77" s="2"/>
     </row>
-    <row r="78" ht="23" customHeight="1" spans="1:20">
+    <row r="78" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A78" s="2" t="s">
         <v>296</v>
       </c>
@@ -10322,7 +10325,7 @@
       <c r="S78" s="2"/>
       <c r="T78" s="2"/>
     </row>
-    <row r="79" ht="23" customHeight="1" spans="1:20">
+    <row r="79" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A79" s="2" t="s">
         <v>299</v>
       </c>
@@ -10378,7 +10381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" ht="23" customHeight="1" spans="1:20">
+    <row r="80" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A80" s="2" t="s">
         <v>301</v>
       </c>
@@ -10480,7 +10483,7 @@
       <c r="S81" s="2"/>
       <c r="T81" s="2"/>
     </row>
-    <row r="82" ht="23" customHeight="1" spans="1:20">
+    <row r="82" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A82" s="2" t="s">
         <v>307</v>
       </c>
@@ -10534,7 +10537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" ht="23" customHeight="1" spans="1:20">
+    <row r="83" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A83" s="2" t="s">
         <v>309</v>
       </c>
@@ -10584,7 +10587,7 @@
       <c r="S83" s="2"/>
       <c r="T83" s="2"/>
     </row>
-    <row r="84" ht="23" customHeight="1" spans="1:20">
+    <row r="84" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A84" s="2" t="s">
         <v>312</v>
       </c>
@@ -10634,7 +10637,7 @@
       <c r="S84" s="2"/>
       <c r="T84" s="2"/>
     </row>
-    <row r="85" ht="23" customHeight="1" spans="1:20">
+    <row r="85" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A85" s="2" t="s">
         <v>315</v>
       </c>
@@ -10688,7 +10691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" ht="23" customHeight="1" spans="1:20">
+    <row r="86" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A86" s="2" t="s">
         <v>320</v>
       </c>
@@ -10794,7 +10797,7 @@
       </c>
       <c r="T87" s="2"/>
     </row>
-    <row r="88" ht="23" customHeight="1" spans="1:20">
+    <row r="88" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A88" s="2" t="s">
         <v>325</v>
       </c>
@@ -10846,7 +10849,7 @@
       <c r="S88" s="2"/>
       <c r="T88" s="2"/>
     </row>
-    <row r="89" ht="23" customHeight="1" spans="1:20">
+    <row r="89" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A89" s="2" t="s">
         <v>329</v>
       </c>
@@ -10900,7 +10903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" ht="23" customHeight="1" spans="1:20">
+    <row r="90" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A90" s="2" t="s">
         <v>332</v>
       </c>
@@ -10950,7 +10953,7 @@
       <c r="S90" s="2"/>
       <c r="T90" s="2"/>
     </row>
-    <row r="91" ht="23" customHeight="1" spans="1:20">
+    <row r="91" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A91" s="2" t="s">
         <v>335</v>
       </c>
@@ -11000,7 +11003,7 @@
       <c r="S91" s="2"/>
       <c r="T91" s="2"/>
     </row>
-    <row r="92" ht="23" customHeight="1" spans="1:20">
+    <row r="92" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A92" s="2" t="s">
         <v>337</v>
       </c>
@@ -11056,7 +11059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" ht="23" customHeight="1" spans="1:20">
+    <row r="93" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A93" s="2" t="s">
         <v>339</v>
       </c>
@@ -11110,7 +11113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" ht="23" customHeight="1" spans="1:20">
+    <row r="94" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A94" s="2" t="s">
         <v>342</v>
       </c>
@@ -11162,7 +11165,7 @@
       <c r="S94" s="2"/>
       <c r="T94" s="2"/>
     </row>
-    <row r="95" ht="23" customHeight="1" spans="1:20">
+    <row r="95" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A95" s="2" t="s">
         <v>345</v>
       </c>
@@ -11216,7 +11219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" ht="23" customHeight="1" spans="1:20">
+    <row r="96" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A96" s="2" t="s">
         <v>348</v>
       </c>
@@ -11270,7 +11273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" ht="23" customHeight="1" spans="1:20">
+    <row r="97" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A97" s="2" t="s">
         <v>352</v>
       </c>
@@ -11320,7 +11323,7 @@
       <c r="S97" s="2"/>
       <c r="T97" s="2"/>
     </row>
-    <row r="98" ht="23" customHeight="1" spans="1:20">
+    <row r="98" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A98" s="2" t="s">
         <v>353</v>
       </c>
@@ -11428,7 +11431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" ht="23" customHeight="1" spans="1:20">
+    <row r="100" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A100" s="2" t="s">
         <v>359</v>
       </c>
@@ -11478,7 +11481,7 @@
       <c r="S100" s="2"/>
       <c r="T100" s="2"/>
     </row>
-    <row r="101" ht="23" customHeight="1" spans="1:20">
+    <row r="101" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A101" s="2" t="s">
         <v>362</v>
       </c>
@@ -11532,7 +11535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" ht="23" customHeight="1" spans="1:20">
+    <row r="102" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A102" s="2" t="s">
         <v>364</v>
       </c>
@@ -11584,7 +11587,7 @@
       <c r="S102" s="2"/>
       <c r="T102" s="2"/>
     </row>
-    <row r="103" ht="23" customHeight="1" spans="1:20">
+    <row r="103" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A103" s="2" t="s">
         <v>366</v>
       </c>
@@ -11634,7 +11637,7 @@
       <c r="S103" s="2"/>
       <c r="T103" s="2"/>
     </row>
-    <row r="104" ht="23" customHeight="1" spans="1:20">
+    <row r="104" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A104" s="2" t="s">
         <v>369</v>
       </c>
@@ -11686,7 +11689,7 @@
       </c>
       <c r="T104" s="2"/>
     </row>
-    <row r="105" ht="23" customHeight="1" spans="1:20">
+    <row r="105" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A105" s="2" t="s">
         <v>372</v>
       </c>
@@ -11740,7 +11743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" ht="23" customHeight="1" spans="1:20">
+    <row r="106" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A106" s="2" t="s">
         <v>376</v>
       </c>
@@ -11796,7 +11799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" ht="23" customHeight="1" spans="1:20">
+    <row r="107" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A107" s="2" t="s">
         <v>379</v>
       </c>
@@ -11852,7 +11855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" ht="23" customHeight="1" spans="1:20">
+    <row r="108" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A108" s="2" t="s">
         <v>381</v>
       </c>
@@ -11908,7 +11911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" ht="23" customHeight="1" spans="1:20">
+    <row r="109" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A109" s="2" t="s">
         <v>382</v>
       </c>
@@ -11964,7 +11967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" ht="23" customHeight="1" spans="1:20">
+    <row r="110" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A110" s="2" t="s">
         <v>384</v>
       </c>
@@ -12076,7 +12079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" ht="23" customHeight="1" spans="1:20">
+    <row r="112" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A112" s="2" t="s">
         <v>390</v>
       </c>
@@ -12130,7 +12133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" ht="23" customHeight="1" spans="1:20">
+    <row r="113" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A113" s="2" t="s">
         <v>393</v>
       </c>
@@ -12184,7 +12187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" ht="23" customHeight="1" spans="1:20">
+    <row r="114" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A114" s="2" t="s">
         <v>396</v>
       </c>
@@ -12234,7 +12237,7 @@
       <c r="S114" s="2"/>
       <c r="T114" s="2"/>
     </row>
-    <row r="115" ht="23" customHeight="1" spans="1:20">
+    <row r="115" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A115" s="2" t="s">
         <v>399</v>
       </c>
@@ -12288,7 +12291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" ht="23" customHeight="1" spans="1:20">
+    <row r="116" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A116" s="2" t="s">
         <v>401</v>
       </c>
@@ -12388,7 +12391,7 @@
       <c r="S117" s="2"/>
       <c r="T117" s="2"/>
     </row>
-    <row r="118" ht="23" customHeight="1" spans="1:20">
+    <row r="118" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A118" s="2" t="s">
         <v>407</v>
       </c>
@@ -12442,7 +12445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" ht="23" customHeight="1" spans="1:20">
+    <row r="119" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A119" s="2" t="s">
         <v>409</v>
       </c>
@@ -12494,7 +12497,7 @@
       <c r="S119" s="2"/>
       <c r="T119" s="2"/>
     </row>
-    <row r="120" ht="23" customHeight="1" spans="1:20">
+    <row r="120" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A120" s="2" t="s">
         <v>411</v>
       </c>
@@ -12548,7 +12551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" ht="23" customHeight="1" spans="1:20">
+    <row r="121" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A121" s="2" t="s">
         <v>413</v>
       </c>
@@ -12656,7 +12659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" ht="23" customHeight="1" spans="1:20">
+    <row r="123" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A123" s="2" t="s">
         <v>417</v>
       </c>
@@ -12706,7 +12709,7 @@
       <c r="S123" s="2"/>
       <c r="T123" s="2"/>
     </row>
-    <row r="124" ht="23" customHeight="1" spans="1:20">
+    <row r="124" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A124" s="2" t="s">
         <v>421</v>
       </c>
@@ -12762,7 +12765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" ht="23" customHeight="1" spans="1:20">
+    <row r="125" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A125" s="2" t="s">
         <v>424</v>
       </c>
@@ -12818,7 +12821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" ht="23" customHeight="1" spans="1:20">
+    <row r="126" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A126" s="2" t="s">
         <v>427</v>
       </c>
@@ -12926,7 +12929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" ht="23" customHeight="1" spans="1:20">
+    <row r="128" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A128" s="2" t="s">
         <v>434</v>
       </c>
@@ -12980,7 +12983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" ht="23" customHeight="1" spans="1:20">
+    <row r="129" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A129" s="2" t="s">
         <v>436</v>
       </c>
@@ -13030,7 +13033,7 @@
       <c r="S129" s="2"/>
       <c r="T129" s="2"/>
     </row>
-    <row r="130" ht="23" customHeight="1" spans="1:20">
+    <row r="130" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A130" s="2" t="s">
         <v>440</v>
       </c>
@@ -13084,7 +13087,7 @@
       </c>
       <c r="T130" s="2"/>
     </row>
-    <row r="131" ht="23" customHeight="1" spans="1:20">
+    <row r="131" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A131" s="2" t="s">
         <v>442</v>
       </c>
@@ -13194,7 +13197,7 @@
       </c>
       <c r="T132" s="2"/>
     </row>
-    <row r="133" ht="23" customHeight="1" spans="1:20">
+    <row r="133" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A133" s="2" t="s">
         <v>448</v>
       </c>
@@ -13250,7 +13253,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" ht="23" customHeight="1" spans="1:20">
+    <row r="134" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A134" s="2" t="s">
         <v>450</v>
       </c>
@@ -13304,7 +13307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" ht="23" customHeight="1" spans="1:20">
+    <row r="135" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A135" s="2" t="s">
         <v>453</v>
       </c>
@@ -13354,7 +13357,7 @@
       <c r="S135" s="2"/>
       <c r="T135" s="2"/>
     </row>
-    <row r="136" ht="23" customHeight="1" spans="1:20">
+    <row r="136" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A136" s="2" t="s">
         <v>456</v>
       </c>
@@ -13462,7 +13465,7 @@
       </c>
       <c r="T137" s="2"/>
     </row>
-    <row r="138" ht="23" customHeight="1" spans="1:20">
+    <row r="138" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A138" s="2" t="s">
         <v>463</v>
       </c>
@@ -13514,7 +13517,7 @@
       </c>
       <c r="T138" s="2"/>
     </row>
-    <row r="139" ht="23" customHeight="1" spans="1:20">
+    <row r="139" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A139" s="2" t="s">
         <v>466</v>
       </c>
@@ -13566,7 +13569,7 @@
       <c r="S139" s="2"/>
       <c r="T139" s="2"/>
     </row>
-    <row r="140" ht="23" customHeight="1" spans="1:20">
+    <row r="140" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A140" s="2" t="s">
         <v>468</v>
       </c>
@@ -13622,7 +13625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" ht="23" customHeight="1" spans="1:20">
+    <row r="141" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A141" s="2" t="s">
         <v>470</v>
       </c>
@@ -13730,7 +13733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" ht="23" customHeight="1" spans="1:20">
+    <row r="143" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A143" s="2" t="s">
         <v>474</v>
       </c>
@@ -13780,7 +13783,7 @@
       <c r="S143" s="2"/>
       <c r="T143" s="2"/>
     </row>
-    <row r="144" ht="23" customHeight="1" spans="1:20">
+    <row r="144" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A144" s="2" t="s">
         <v>477</v>
       </c>
@@ -13832,7 +13835,7 @@
       <c r="S144" s="2"/>
       <c r="T144" s="2"/>
     </row>
-    <row r="145" ht="23" customHeight="1" spans="1:20">
+    <row r="145" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A145" s="2" t="s">
         <v>480</v>
       </c>
@@ -13886,7 +13889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" ht="23" customHeight="1" spans="1:20">
+    <row r="146" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A146" s="2" t="s">
         <v>483</v>
       </c>
@@ -13990,7 +13993,7 @@
       </c>
       <c r="T147" s="2"/>
     </row>
-    <row r="148" ht="23" customHeight="1" spans="1:20">
+    <row r="148" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A148" s="2" t="s">
         <v>489</v>
       </c>
@@ -14044,7 +14047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" ht="23" customHeight="1" spans="1:20">
+    <row r="149" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A149" s="2" t="s">
         <v>491</v>
       </c>
@@ -14098,7 +14101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" ht="23" customHeight="1" spans="1:20">
+    <row r="150" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A150" s="2" t="s">
         <v>495</v>
       </c>
@@ -14154,7 +14157,7 @@
       </c>
       <c r="T150" s="2"/>
     </row>
-    <row r="151" ht="23" customHeight="1" spans="1:20">
+    <row r="151" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A151" s="2" t="s">
         <v>498</v>
       </c>
@@ -14264,7 +14267,7 @@
       </c>
       <c r="T152" s="2"/>
     </row>
-    <row r="153" ht="23" customHeight="1" spans="1:20">
+    <row r="153" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A153" s="2" t="s">
         <v>504</v>
       </c>
@@ -14320,7 +14323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" ht="23" customHeight="1" spans="1:20">
+    <row r="154" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A154" s="2" t="s">
         <v>508</v>
       </c>
@@ -14370,7 +14373,7 @@
       <c r="S154" s="2"/>
       <c r="T154" s="2"/>
     </row>
-    <row r="155" ht="23" customHeight="1" spans="1:20">
+    <row r="155" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A155" s="2" t="s">
         <v>511</v>
       </c>
@@ -14426,7 +14429,7 @@
       </c>
       <c r="T155" s="2"/>
     </row>
-    <row r="156" ht="23" customHeight="1" spans="1:20">
+    <row r="156" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A156" s="2" t="s">
         <v>515</v>
       </c>
@@ -14538,7 +14541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" ht="23" customHeight="1" spans="1:20">
+    <row r="158" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A158" s="2" t="s">
         <v>522</v>
       </c>
@@ -14592,7 +14595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" ht="23" customHeight="1" spans="1:20">
+    <row r="159" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A159" s="2" t="s">
         <v>525</v>
       </c>
@@ -14646,7 +14649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" ht="23" customHeight="1" spans="1:20">
+    <row r="160" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A160" s="2" t="s">
         <v>528</v>
       </c>
@@ -14698,7 +14701,7 @@
       <c r="S160" s="2"/>
       <c r="T160" s="2"/>
     </row>
-    <row r="161" ht="23" customHeight="1" spans="1:20">
+    <row r="161" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A161" s="2" t="s">
         <v>532</v>
       </c>
@@ -14808,7 +14811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" ht="23" customHeight="1" spans="1:20">
+    <row r="163" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A163" s="2" t="s">
         <v>537</v>
       </c>
@@ -14864,7 +14867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" ht="23" customHeight="1" spans="1:20">
+    <row r="164" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A164" s="2" t="s">
         <v>539</v>
       </c>
@@ -14918,7 +14921,7 @@
       </c>
       <c r="T164" s="2"/>
     </row>
-    <row r="165" ht="23" customHeight="1" spans="1:20">
+    <row r="165" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A165" s="2" t="s">
         <v>544</v>
       </c>
@@ -14968,7 +14971,7 @@
       <c r="S165" s="2"/>
       <c r="T165" s="2"/>
     </row>
-    <row r="166" ht="23" customHeight="1" spans="1:20">
+    <row r="166" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A166" s="2" t="s">
         <v>547</v>
       </c>
@@ -15078,7 +15081,7 @@
       </c>
       <c r="T167" s="2"/>
     </row>
-    <row r="168" ht="23" customHeight="1" spans="1:20">
+    <row r="168" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A168" s="2" t="s">
         <v>552</v>
       </c>
@@ -15130,7 +15133,7 @@
       <c r="S168" s="2"/>
       <c r="T168" s="2"/>
     </row>
-    <row r="169" ht="23" customHeight="1" spans="1:20">
+    <row r="169" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A169" s="2" t="s">
         <v>555</v>
       </c>
@@ -15186,7 +15189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" ht="23" customHeight="1" spans="1:20">
+    <row r="170" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A170" s="2" t="s">
         <v>557</v>
       </c>
@@ -15236,7 +15239,7 @@
       <c r="S170" s="2"/>
       <c r="T170" s="2"/>
     </row>
-    <row r="171" ht="23" customHeight="1" spans="1:20">
+    <row r="171" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A171" s="2" t="s">
         <v>560</v>
       </c>
@@ -15344,7 +15347,7 @@
       </c>
       <c r="T172" s="2"/>
     </row>
-    <row r="173" ht="23" customHeight="1" spans="1:20">
+    <row r="173" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A173" s="2" t="s">
         <v>566</v>
       </c>
@@ -15396,7 +15399,7 @@
       <c r="S173" s="2"/>
       <c r="T173" s="2"/>
     </row>
-    <row r="174" ht="23" customHeight="1" spans="1:20">
+    <row r="174" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A174" s="2" t="s">
         <v>568</v>
       </c>
@@ -15452,7 +15455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" ht="23" customHeight="1" spans="1:20">
+    <row r="175" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A175" s="2" t="s">
         <v>571</v>
       </c>
@@ -15502,7 +15505,7 @@
       <c r="S175" s="2"/>
       <c r="T175" s="2"/>
     </row>
-    <row r="176" ht="23" customHeight="1" spans="1:20">
+    <row r="176" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A176" s="2" t="s">
         <v>573</v>
       </c>
@@ -15606,7 +15609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" ht="23" customHeight="1" spans="1:20">
+    <row r="178" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A178" s="2" t="s">
         <v>578</v>
       </c>
@@ -15660,7 +15663,7 @@
       <c r="S178" s="2"/>
       <c r="T178" s="2"/>
     </row>
-    <row r="179" ht="23" customHeight="1" spans="1:20">
+    <row r="179" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A179" s="2" t="s">
         <v>581</v>
       </c>
@@ -15710,7 +15713,7 @@
       <c r="S179" s="2"/>
       <c r="T179" s="2"/>
     </row>
-    <row r="180" ht="23" customHeight="1" spans="1:20">
+    <row r="180" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A180" s="2" t="s">
         <v>584</v>
       </c>
@@ -15766,7 +15769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" ht="23" customHeight="1" spans="1:20">
+    <row r="181" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A181" s="2" t="s">
         <v>587</v>
       </c>
@@ -15874,7 +15877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" ht="23" customHeight="1" spans="1:20">
+    <row r="183" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A183" s="2" t="s">
         <v>591</v>
       </c>
@@ -15926,7 +15929,7 @@
       <c r="S183" s="2"/>
       <c r="T183" s="2"/>
     </row>
-    <row r="184" ht="23" customHeight="1" spans="1:20">
+    <row r="184" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A184" s="2" t="s">
         <v>593</v>
       </c>
@@ -15980,7 +15983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" ht="23" customHeight="1" spans="1:20">
+    <row r="185" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A185" s="2" t="s">
         <v>596</v>
       </c>
@@ -16030,7 +16033,7 @@
       <c r="S185" s="2"/>
       <c r="T185" s="2"/>
     </row>
-    <row r="186" ht="23" customHeight="1" spans="1:20">
+    <row r="186" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A186" s="2" t="s">
         <v>598</v>
       </c>
@@ -16136,7 +16139,7 @@
       <c r="S187" s="2"/>
       <c r="T187" s="2"/>
     </row>
-    <row r="188" ht="23" customHeight="1" spans="1:20">
+    <row r="188" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A188" s="2" t="s">
         <v>603</v>
       </c>
@@ -16186,7 +16189,7 @@
       <c r="S188" s="2"/>
       <c r="T188" s="2"/>
     </row>
-    <row r="189" ht="23" customHeight="1" spans="1:20">
+    <row r="189" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A189" s="2" t="s">
         <v>605</v>
       </c>
@@ -16240,7 +16243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" ht="23" customHeight="1" spans="1:20">
+    <row r="190" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A190" s="2" t="s">
         <v>606</v>
       </c>
@@ -16294,7 +16297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" ht="23" customHeight="1" spans="1:20">
+    <row r="191" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A191" s="2" t="s">
         <v>609</v>
       </c>
@@ -16394,7 +16397,7 @@
       <c r="S192" s="2"/>
       <c r="T192" s="2"/>
     </row>
-    <row r="193" ht="23" customHeight="1" spans="1:20">
+    <row r="193" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A193" s="2" t="s">
         <v>613</v>
       </c>
@@ -16446,7 +16449,7 @@
       <c r="S193" s="2"/>
       <c r="T193" s="2"/>
     </row>
-    <row r="194" ht="23" customHeight="1" spans="1:20">
+    <row r="194" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A194" s="2" t="s">
         <v>617</v>
       </c>
@@ -16500,7 +16503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" ht="23" customHeight="1" spans="1:20">
+    <row r="195" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A195" s="2" t="s">
         <v>619</v>
       </c>
@@ -16552,7 +16555,7 @@
       <c r="S195" s="2"/>
       <c r="T195" s="2"/>
     </row>
-    <row r="196" ht="23" customHeight="1" spans="1:20">
+    <row r="196" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A196" s="2" t="s">
         <v>622</v>
       </c>
@@ -16656,7 +16659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" ht="23" customHeight="1" spans="1:20">
+    <row r="198" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A198" s="2" t="s">
         <v>629</v>
       </c>
@@ -16710,7 +16713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" ht="23" customHeight="1" spans="1:20">
+    <row r="199" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A199" s="2" t="s">
         <v>632</v>
       </c>
@@ -16760,7 +16763,7 @@
       <c r="S199" s="2"/>
       <c r="T199" s="2"/>
     </row>
-    <row r="200" ht="23" customHeight="1" spans="1:20">
+    <row r="200" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A200" s="2" t="s">
         <v>634</v>
       </c>
@@ -16810,7 +16813,7 @@
       <c r="S200" s="2"/>
       <c r="T200" s="2"/>
     </row>
-    <row r="201" ht="23" customHeight="1" spans="1:20">
+    <row r="201" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A201" s="2" t="s">
         <v>637</v>
       </c>
@@ -16916,7 +16919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" ht="23" customHeight="1" spans="1:20">
+    <row r="203" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A203" s="2" t="s">
         <v>641</v>
       </c>
@@ -16966,7 +16969,7 @@
       <c r="S203" s="2"/>
       <c r="T203" s="2"/>
     </row>
-    <row r="204" ht="23" customHeight="1" spans="1:20">
+    <row r="204" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A204" s="2" t="s">
         <v>644</v>
       </c>
@@ -17020,7 +17023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" ht="23" customHeight="1" spans="1:20">
+    <row r="205" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A205" s="2" t="s">
         <v>645</v>
       </c>
@@ -17074,7 +17077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" ht="23" customHeight="1" spans="1:20">
+    <row r="206" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A206" s="2" t="s">
         <v>648</v>
       </c>
@@ -17184,7 +17187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" ht="23" customHeight="1" spans="1:20">
+    <row r="208" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A208" s="2" t="s">
         <v>652</v>
       </c>
@@ -17236,7 +17239,7 @@
       <c r="S208" s="2"/>
       <c r="T208" s="2"/>
     </row>
-    <row r="209" ht="23" customHeight="1" spans="1:20">
+    <row r="209" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A209" s="2" t="s">
         <v>655</v>
       </c>
@@ -17290,7 +17293,7 @@
       </c>
       <c r="T209" s="2"/>
     </row>
-    <row r="210" ht="23" customHeight="1" spans="1:20">
+    <row r="210" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A210" s="2" t="s">
         <v>657</v>
       </c>
@@ -17344,7 +17347,7 @@
       </c>
       <c r="T210" s="2"/>
     </row>
-    <row r="211" ht="23" customHeight="1" spans="1:20">
+    <row r="211" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A211" s="2" t="s">
         <v>659</v>
       </c>
@@ -17452,7 +17455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" ht="23" customHeight="1" spans="1:20">
+    <row r="213" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A213" s="2" t="s">
         <v>664</v>
       </c>
@@ -17502,7 +17505,7 @@
       <c r="S213" s="2"/>
       <c r="T213" s="2"/>
     </row>
-    <row r="214" ht="23" customHeight="1" spans="1:20">
+    <row r="214" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A214" s="2" t="s">
         <v>666</v>
       </c>
@@ -17558,7 +17561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" ht="23" customHeight="1" spans="1:20">
+    <row r="215" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A215" s="2" t="s">
         <v>668</v>
       </c>
@@ -17614,7 +17617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" ht="23" customHeight="1" spans="1:20">
+    <row r="216" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A216" s="2" t="s">
         <v>670</v>
       </c>
@@ -17724,7 +17727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" ht="23" customHeight="1" spans="1:20">
+    <row r="218" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A218" s="2" t="s">
         <v>674</v>
       </c>
@@ -17776,7 +17779,7 @@
       <c r="S218" s="2"/>
       <c r="T218" s="2"/>
     </row>
-    <row r="219" ht="23" customHeight="1" spans="1:20">
+    <row r="219" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A219" s="2" t="s">
         <v>677</v>
       </c>
@@ -17826,7 +17829,7 @@
       <c r="S219" s="2"/>
       <c r="T219" s="2"/>
     </row>
-    <row r="220" ht="23" customHeight="1" spans="1:20">
+    <row r="220" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A220" s="2" t="s">
         <v>679</v>
       </c>
@@ -17876,7 +17879,7 @@
       <c r="S220" s="2"/>
       <c r="T220" s="2"/>
     </row>
-    <row r="221" ht="23" customHeight="1" spans="1:20">
+    <row r="221" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A221" s="2" t="s">
         <v>682</v>
       </c>
@@ -17980,7 +17983,7 @@
       <c r="S222" s="2"/>
       <c r="T222" s="2"/>
     </row>
-    <row r="223" ht="23" customHeight="1" spans="1:20">
+    <row r="223" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A223" s="2" t="s">
         <v>687</v>
       </c>
@@ -18034,7 +18037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" ht="23" customHeight="1" spans="1:20">
+    <row r="224" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A224" s="2" t="s">
         <v>689</v>
       </c>
@@ -18084,7 +18087,7 @@
       <c r="S224" s="2"/>
       <c r="T224" s="2"/>
     </row>
-    <row r="225" ht="23" customHeight="1" spans="1:20">
+    <row r="225" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A225" s="2" t="s">
         <v>691</v>
       </c>
@@ -18138,7 +18141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" ht="23" customHeight="1" spans="1:20">
+    <row r="226" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A226" s="2" t="s">
         <v>694</v>
       </c>
@@ -18246,7 +18249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" ht="23" customHeight="1" spans="1:20">
+    <row r="228" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A228" s="2" t="s">
         <v>701</v>
       </c>
@@ -18302,7 +18305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" ht="23" customHeight="1" spans="1:20">
+    <row r="229" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A229" s="2" t="s">
         <v>704</v>
       </c>
@@ -18356,7 +18359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" ht="23" customHeight="1" spans="1:20">
+    <row r="230" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A230" s="2" t="s">
         <v>706</v>
       </c>
@@ -18412,7 +18415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" ht="23" customHeight="1" spans="1:20">
+    <row r="231" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A231" s="2" t="s">
         <v>708</v>
       </c>
@@ -18522,7 +18525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" ht="23" customHeight="1" spans="1:20">
+    <row r="233" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A233" s="2" t="s">
         <v>713</v>
       </c>
@@ -18576,7 +18579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" ht="23" customHeight="1" spans="1:20">
+    <row r="234" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A234" s="2" t="s">
         <v>716</v>
       </c>
@@ -18628,7 +18631,7 @@
       <c r="S234" s="2"/>
       <c r="T234" s="2"/>
     </row>
-    <row r="235" ht="23" customHeight="1" spans="1:20">
+    <row r="235" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A235" s="2" t="s">
         <v>718</v>
       </c>
@@ -18684,7 +18687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" ht="23" customHeight="1" spans="1:20">
+    <row r="236" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A236" s="2" t="s">
         <v>721</v>
       </c>
@@ -18796,7 +18799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238" ht="23" customHeight="1" spans="1:20">
+    <row r="238" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A238" s="2" t="s">
         <v>728</v>
       </c>
@@ -18850,7 +18853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" ht="23" customHeight="1" spans="1:20">
+    <row r="239" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A239" s="2" t="s">
         <v>730</v>
       </c>
@@ -18902,7 +18905,7 @@
       </c>
       <c r="T239" s="2"/>
     </row>
-    <row r="240" ht="23" customHeight="1" spans="1:20">
+    <row r="240" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A240" s="2" t="s">
         <v>733</v>
       </c>
@@ -18956,7 +18959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" ht="23" customHeight="1" spans="1:20">
+    <row r="241" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A241" s="2" t="s">
         <v>735</v>
       </c>
@@ -19012,7 +19015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="242" ht="23" customHeight="1" spans="1:20">
+    <row r="242" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A242" s="2" t="s">
         <v>736</v>
       </c>
@@ -19068,7 +19071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" ht="23" customHeight="1" spans="1:20">
+    <row r="243" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A243" s="2" t="s">
         <v>740</v>
       </c>
@@ -19120,7 +19123,7 @@
       <c r="S243" s="2"/>
       <c r="T243" s="2"/>
     </row>
-    <row r="244" ht="23" customHeight="1" spans="1:20">
+    <row r="244" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A244" s="2" t="s">
         <v>742</v>
       </c>
@@ -19170,7 +19173,7 @@
       <c r="S244" s="2"/>
       <c r="T244" s="2"/>
     </row>
-    <row r="245" ht="23" customHeight="1" spans="1:20">
+    <row r="245" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A245" s="2" t="s">
         <v>745</v>
       </c>
@@ -19224,7 +19227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" ht="23" customHeight="1" spans="1:20">
+    <row r="246" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A246" s="2" t="s">
         <v>748</v>
       </c>
@@ -19336,7 +19339,7 @@
       </c>
       <c r="T247" s="2"/>
     </row>
-    <row r="248" ht="23" customHeight="1" spans="1:20">
+    <row r="248" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A248" s="2" t="s">
         <v>753</v>
       </c>
@@ -19392,7 +19395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" ht="23" customHeight="1" spans="1:20">
+    <row r="249" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A249" s="2" t="s">
         <v>754</v>
       </c>
@@ -19448,7 +19451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="250" ht="23" customHeight="1" spans="1:20">
+    <row r="250" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A250" s="2" t="s">
         <v>755</v>
       </c>
@@ -19504,7 +19507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" ht="23" customHeight="1" spans="1:20">
+    <row r="251" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A251" s="2" t="s">
         <v>757</v>
       </c>
@@ -19610,7 +19613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="253" ht="23" customHeight="1" spans="1:20">
+    <row r="253" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A253" s="2" t="s">
         <v>760</v>
       </c>
@@ -19664,7 +19667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" ht="23" customHeight="1" spans="1:20">
+    <row r="254" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A254" s="2" t="s">
         <v>763</v>
       </c>
@@ -19714,7 +19717,7 @@
       <c r="S254" s="2"/>
       <c r="T254" s="2"/>
     </row>
-    <row r="255" ht="23" customHeight="1" spans="1:20">
+    <row r="255" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A255" s="2" t="s">
         <v>766</v>
       </c>
@@ -19768,7 +19771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" ht="23" customHeight="1" spans="1:20">
+    <row r="256" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A256" s="2" t="s">
         <v>767</v>
       </c>
@@ -19874,7 +19877,7 @@
       <c r="S257" s="2"/>
       <c r="T257" s="2"/>
     </row>
-    <row r="258" ht="23" customHeight="1" spans="1:20">
+    <row r="258" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A258" s="2" t="s">
         <v>771</v>
       </c>
@@ -19930,7 +19933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" ht="23" customHeight="1" spans="1:20">
+    <row r="259" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A259" s="2" t="s">
         <v>772</v>
       </c>
@@ -19982,7 +19985,7 @@
       <c r="S259" s="2"/>
       <c r="T259" s="2"/>
     </row>
-    <row r="260" ht="23" customHeight="1" spans="1:20">
+    <row r="260" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A260" s="2" t="s">
         <v>773</v>
       </c>
@@ -20034,7 +20037,7 @@
       <c r="S260" s="2"/>
       <c r="T260" s="2"/>
     </row>
-    <row r="261" ht="23" customHeight="1" spans="1:20">
+    <row r="261" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A261" s="2" t="s">
         <v>774</v>
       </c>
@@ -20142,7 +20145,7 @@
       <c r="S262" s="2"/>
       <c r="T262" s="2"/>
     </row>
-    <row r="263" ht="23" customHeight="1" spans="1:20">
+    <row r="263" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A263" s="2" t="s">
         <v>778</v>
       </c>
@@ -20200,7 +20203,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="264" ht="23" customHeight="1" spans="1:20">
+    <row r="264" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A264" s="2" t="s">
         <v>781</v>
       </c>
@@ -20252,7 +20255,7 @@
       </c>
       <c r="T264" s="2"/>
     </row>
-    <row r="265" ht="23" customHeight="1" spans="1:20">
+    <row r="265" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A265" s="2" t="s">
         <v>784</v>
       </c>
@@ -20302,7 +20305,7 @@
       <c r="S265" s="2"/>
       <c r="T265" s="2"/>
     </row>
-    <row r="266" ht="23" customHeight="1" spans="1:20">
+    <row r="266" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A266" s="2" t="s">
         <v>787</v>
       </c>
@@ -20404,7 +20407,7 @@
       <c r="S267" s="2"/>
       <c r="T267" s="2"/>
     </row>
-    <row r="268" ht="23" customHeight="1" spans="1:20">
+    <row r="268" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A268" s="2" t="s">
         <v>793</v>
       </c>
@@ -20460,7 +20463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="269" ht="23" customHeight="1" spans="1:20">
+    <row r="269" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A269" s="2" t="s">
         <v>796</v>
       </c>
@@ -20510,7 +20513,7 @@
       <c r="S269" s="2"/>
       <c r="T269" s="2"/>
     </row>
-    <row r="270" ht="23" customHeight="1" spans="1:20">
+    <row r="270" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A270" s="2" t="s">
         <v>798</v>
       </c>
@@ -20566,7 +20569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271" ht="23" customHeight="1" spans="1:20">
+    <row r="271" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A271" s="2" t="s">
         <v>800</v>
       </c>
@@ -20672,7 +20675,7 @@
       <c r="S272" s="2"/>
       <c r="T272" s="2"/>
     </row>
-    <row r="273" ht="23" customHeight="1" spans="1:20">
+    <row r="273" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A273" s="2" t="s">
         <v>806</v>
       </c>
@@ -20728,7 +20731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="274" ht="23" customHeight="1" spans="1:20">
+    <row r="274" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A274" s="2" t="s">
         <v>809</v>
       </c>
@@ -20782,7 +20785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" ht="23" customHeight="1" spans="1:20">
+    <row r="275" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A275" s="2" t="s">
         <v>811</v>
       </c>
@@ -20832,7 +20835,7 @@
       <c r="S275" s="2"/>
       <c r="T275" s="2"/>
     </row>
-    <row r="276" ht="23" customHeight="1" spans="1:20">
+    <row r="276" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A276" s="2" t="s">
         <v>814</v>
       </c>
@@ -20942,7 +20945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278" ht="23" customHeight="1" spans="1:20">
+    <row r="278" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A278" s="2" t="s">
         <v>819</v>
       </c>
@@ -20996,7 +20999,7 @@
       </c>
       <c r="T278" s="2"/>
     </row>
-    <row r="279" ht="23" customHeight="1" spans="1:20">
+    <row r="279" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A279" s="2" t="s">
         <v>821</v>
       </c>
@@ -21050,7 +21053,7 @@
       </c>
       <c r="T279" s="2"/>
     </row>
-    <row r="280" ht="23" customHeight="1" spans="1:20">
+    <row r="280" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A280" s="2" t="s">
         <v>824</v>
       </c>
@@ -21106,7 +21109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="281" ht="23" customHeight="1" spans="1:20">
+    <row r="281" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A281" s="2" t="s">
         <v>827</v>
       </c>
@@ -21212,7 +21215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="283" ht="23" customHeight="1" spans="1:20">
+    <row r="283" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A283" s="2" t="s">
         <v>833</v>
       </c>
@@ -21266,7 +21269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" ht="23" customHeight="1" spans="1:20">
+    <row r="284" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A284" s="2" t="s">
         <v>835</v>
       </c>
@@ -21320,7 +21323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" ht="23" customHeight="1" spans="1:20">
+    <row r="285" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A285" s="2" t="s">
         <v>838</v>
       </c>
@@ -21374,7 +21377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" ht="23" customHeight="1" spans="1:20">
+    <row r="286" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A286" s="2" t="s">
         <v>841</v>
       </c>
@@ -21486,7 +21489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" ht="23" customHeight="1" spans="1:20">
+    <row r="288" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A288" s="2" t="s">
         <v>845</v>
       </c>
@@ -21540,7 +21543,7 @@
       </c>
       <c r="T288" s="2"/>
     </row>
-    <row r="289" ht="23" customHeight="1" spans="1:20">
+    <row r="289" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A289" s="2" t="s">
         <v>847</v>
       </c>
@@ -21590,7 +21593,7 @@
       <c r="S289" s="2"/>
       <c r="T289" s="2"/>
     </row>
-    <row r="290" ht="23" customHeight="1" spans="1:20">
+    <row r="290" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A290" s="2" t="s">
         <v>850</v>
       </c>
@@ -21646,7 +21649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="291" ht="23" customHeight="1" spans="1:20">
+    <row r="291" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A291" s="2" t="s">
         <v>852</v>
       </c>
@@ -21750,7 +21753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" ht="23" customHeight="1" spans="1:20">
+    <row r="293" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A293" s="2" t="s">
         <v>859</v>
       </c>
@@ -21806,7 +21809,7 @@
       </c>
       <c r="T293" s="2"/>
     </row>
-    <row r="294" ht="23" customHeight="1" spans="1:20">
+    <row r="294" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A294" s="2" t="s">
         <v>861</v>
       </c>
@@ -21856,7 +21859,7 @@
       <c r="S294" s="2"/>
       <c r="T294" s="2"/>
     </row>
-    <row r="295" ht="23" customHeight="1" spans="1:20">
+    <row r="295" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A295" s="2" t="s">
         <v>864</v>
       </c>
@@ -21910,7 +21913,7 @@
       </c>
       <c r="T295" s="2"/>
     </row>
-    <row r="296" ht="23" customHeight="1" spans="1:20">
+    <row r="296" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A296" s="2" t="s">
         <v>866</v>
       </c>
@@ -22014,7 +22017,7 @@
       <c r="S297" s="2"/>
       <c r="T297" s="2"/>
     </row>
-    <row r="298" ht="23" customHeight="1" spans="1:20">
+    <row r="298" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A298" s="2" t="s">
         <v>869</v>
       </c>
@@ -22068,7 +22071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" ht="23" customHeight="1" spans="1:20">
+    <row r="299" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A299" s="2" t="s">
         <v>870</v>
       </c>
@@ -22124,7 +22127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="300" ht="23" customHeight="1" spans="1:20">
+    <row r="300" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A300" s="2" t="s">
         <v>872</v>
       </c>
@@ -22176,7 +22179,7 @@
       <c r="S300" s="2"/>
       <c r="T300" s="2"/>
     </row>
-    <row r="301" ht="23" customHeight="1" spans="1:20">
+    <row r="301" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A301" s="2" t="s">
         <v>875</v>
       </c>
@@ -22280,7 +22283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" ht="23" customHeight="1" spans="1:20">
+    <row r="303" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A303" s="2" t="s">
         <v>880</v>
       </c>
@@ -22334,7 +22337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" ht="23" customHeight="1" spans="1:20">
+    <row r="304" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A304" s="2" t="s">
         <v>882</v>
       </c>
@@ -22388,7 +22391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" ht="23" customHeight="1" spans="1:20">
+    <row r="305" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A305" s="2" t="s">
         <v>884</v>
       </c>
@@ -22442,7 +22445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" ht="23" customHeight="1" spans="1:20">
+    <row r="306" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A306" s="2" t="s">
         <v>886</v>
       </c>
@@ -22552,7 +22555,7 @@
       </c>
       <c r="T307" s="2"/>
     </row>
-    <row r="308" ht="23" customHeight="1" spans="1:20">
+    <row r="308" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A308" s="2" t="s">
         <v>891</v>
       </c>
@@ -22608,7 +22611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" ht="23" customHeight="1" spans="1:20">
+    <row r="309" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A309" s="2" t="s">
         <v>893</v>
       </c>
@@ -22662,7 +22665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" ht="23" customHeight="1" spans="1:20">
+    <row r="310" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A310" s="2" t="s">
         <v>894</v>
       </c>
@@ -22712,7 +22715,7 @@
       <c r="S310" s="2"/>
       <c r="T310" s="2"/>
     </row>
-    <row r="311" ht="23" customHeight="1" spans="1:20">
+    <row r="311" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A311" s="2" t="s">
         <v>896</v>
       </c>
@@ -22822,7 +22825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="313" ht="23" customHeight="1" spans="1:20">
+    <row r="313" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A313" s="2" t="s">
         <v>900</v>
       </c>
@@ -22872,7 +22875,7 @@
       <c r="S313" s="2"/>
       <c r="T313" s="2"/>
     </row>
-    <row r="314" ht="23" customHeight="1" spans="1:20">
+    <row r="314" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A314" s="2" t="s">
         <v>902</v>
       </c>
@@ -22928,7 +22931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315" ht="23" customHeight="1" spans="1:20">
+    <row r="315" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A315" s="2" t="s">
         <v>903</v>
       </c>
@@ -22984,7 +22987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" ht="23" customHeight="1" spans="1:20">
+    <row r="316" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A316" s="2" t="s">
         <v>905</v>
       </c>
@@ -23090,7 +23093,7 @@
       <c r="S317" s="2"/>
       <c r="T317" s="2"/>
     </row>
-    <row r="318" ht="23" customHeight="1" spans="1:20">
+    <row r="318" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A318" s="2" t="s">
         <v>910</v>
       </c>
@@ -23140,7 +23143,7 @@
       <c r="S318" s="2"/>
       <c r="T318" s="2"/>
     </row>
-    <row r="319" ht="23" customHeight="1" spans="1:20">
+    <row r="319" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A319" s="2" t="s">
         <v>913</v>
       </c>
@@ -23196,7 +23199,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="320" ht="23" customHeight="1" spans="1:20">
+    <row r="320" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A320" s="2" t="s">
         <v>915</v>
       </c>
@@ -23250,7 +23253,7 @@
       </c>
       <c r="T320" s="2"/>
     </row>
-    <row r="321" ht="23" customHeight="1" spans="1:20">
+    <row r="321" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A321" s="2" t="s">
         <v>917</v>
       </c>
@@ -23360,7 +23363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="323" ht="23" customHeight="1" spans="1:20">
+    <row r="323" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A323" s="2" t="s">
         <v>922</v>
       </c>
@@ -23410,7 +23413,7 @@
       <c r="S323" s="2"/>
       <c r="T323" s="2"/>
     </row>
-    <row r="324" ht="23" customHeight="1" spans="1:20">
+    <row r="324" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A324" s="2" t="s">
         <v>925</v>
       </c>
@@ -23464,7 +23467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325" ht="23" customHeight="1" spans="1:20">
+    <row r="325" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A325" s="2" t="s">
         <v>927</v>
       </c>
@@ -23518,7 +23521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="326" ht="23" customHeight="1" spans="1:20">
+    <row r="326" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A326" s="2" t="s">
         <v>929</v>
       </c>
@@ -23628,7 +23631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="328" ht="23" customHeight="1" spans="1:20">
+    <row r="328" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A328" s="2" t="s">
         <v>931</v>
       </c>
@@ -23684,7 +23687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="329" ht="23" customHeight="1" spans="1:20">
+    <row r="329" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A329" s="2" t="s">
         <v>934</v>
       </c>
@@ -23740,7 +23743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" ht="23" customHeight="1" spans="1:20">
+    <row r="330" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A330" s="2" t="s">
         <v>936</v>
       </c>
@@ -23790,7 +23793,7 @@
       <c r="S330" s="2"/>
       <c r="T330" s="2"/>
     </row>
-    <row r="331" ht="23" customHeight="1" spans="1:20">
+    <row r="331" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A331" s="2" t="s">
         <v>939</v>
       </c>
@@ -23900,7 +23903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="333" ht="23" customHeight="1" spans="1:20">
+    <row r="333" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A333" s="2" t="s">
         <v>944</v>
       </c>
@@ -23954,7 +23957,7 @@
       </c>
       <c r="T333" s="2"/>
     </row>
-    <row r="334" ht="23" customHeight="1" spans="1:20">
+    <row r="334" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A334" s="2" t="s">
         <v>947</v>
       </c>
@@ -24010,7 +24013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="335" ht="23" customHeight="1" spans="1:20">
+    <row r="335" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A335" s="2" t="s">
         <v>950</v>
       </c>
@@ -24066,7 +24069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="336" ht="23" customHeight="1" spans="1:20">
+    <row r="336" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A336" s="2" t="s">
         <v>952</v>
       </c>
@@ -24176,7 +24179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="338" ht="23" customHeight="1" spans="1:20">
+    <row r="338" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A338" s="2" t="s">
         <v>954</v>
       </c>
@@ -24234,7 +24237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="339" ht="23" customHeight="1" spans="1:20">
+    <row r="339" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A339" s="2" t="s">
         <v>956</v>
       </c>
@@ -24290,7 +24293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="340" ht="23" customHeight="1" spans="1:20">
+    <row r="340" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A340" s="2" t="s">
         <v>957</v>
       </c>
@@ -24344,7 +24347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="341" ht="23" customHeight="1" spans="1:20">
+    <row r="341" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A341" s="2" t="s">
         <v>959</v>
       </c>
@@ -24454,7 +24457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="343" ht="23" customHeight="1" spans="1:20">
+    <row r="343" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A343" s="2" t="s">
         <v>963</v>
       </c>
@@ -24510,7 +24513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="344" ht="23" customHeight="1" spans="1:20">
+    <row r="344" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A344" s="2" t="s">
         <v>966</v>
       </c>
@@ -24566,7 +24569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="345" ht="23" customHeight="1" spans="1:20">
+    <row r="345" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A345" s="2" t="s">
         <v>969</v>
       </c>
@@ -24622,7 +24625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="346" ht="23" customHeight="1" spans="1:20">
+    <row r="346" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A346" s="2" t="s">
         <v>972</v>
       </c>
@@ -24728,7 +24731,7 @@
       <c r="S347" s="2"/>
       <c r="T347" s="2"/>
     </row>
-    <row r="348" ht="23" customHeight="1" spans="1:20">
+    <row r="348" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A348" s="2" t="s">
         <v>977</v>
       </c>
@@ -24784,7 +24787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="349" ht="23" customHeight="1" spans="1:20">
+    <row r="349" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A349" s="2" t="s">
         <v>978</v>
       </c>
@@ -24836,7 +24839,7 @@
       <c r="S349" s="2"/>
       <c r="T349" s="2"/>
     </row>
-    <row r="350" ht="23" customHeight="1" spans="1:20">
+    <row r="350" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A350" s="2" t="s">
         <v>981</v>
       </c>
@@ -24894,7 +24897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="351" ht="23" customHeight="1" spans="1:20">
+    <row r="351" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A351" s="2" t="s">
         <v>984</v>
       </c>
@@ -25002,7 +25005,7 @@
       </c>
       <c r="T352" s="2"/>
     </row>
-    <row r="353" ht="23" customHeight="1" spans="1:20">
+    <row r="353" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A353" s="2" t="s">
         <v>989</v>
       </c>
@@ -25058,7 +25061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="354" ht="23" customHeight="1" spans="1:20">
+    <row r="354" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A354" s="2" t="s">
         <v>991</v>
       </c>
@@ -25110,7 +25113,7 @@
       <c r="S354" s="2"/>
       <c r="T354" s="2"/>
     </row>
-    <row r="355" ht="23" customHeight="1" spans="1:20">
+    <row r="355" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A355" s="2" t="s">
         <v>993</v>
       </c>
@@ -25164,7 +25167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="356" ht="23" customHeight="1" spans="1:20">
+    <row r="356" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A356" s="2" t="s">
         <v>996</v>
       </c>
@@ -25268,7 +25271,7 @@
       <c r="S357" s="2"/>
       <c r="T357" s="2"/>
     </row>
-    <row r="358" ht="23" customHeight="1" spans="1:20">
+    <row r="358" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A358" s="2" t="s">
         <v>1000</v>
       </c>
@@ -25324,7 +25327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="359" ht="23" customHeight="1" spans="1:20">
+    <row r="359" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A359" s="2" t="s">
         <v>1002</v>
       </c>
@@ -25380,7 +25383,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="360" ht="23" customHeight="1" spans="1:20">
+    <row r="360" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A360" s="2" t="s">
         <v>1004</v>
       </c>
@@ -25432,7 +25435,7 @@
       <c r="S360" s="2"/>
       <c r="T360" s="2"/>
     </row>
-    <row r="361" ht="23" customHeight="1" spans="1:20">
+    <row r="361" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A361" s="2" t="s">
         <v>1007</v>
       </c>
@@ -25542,7 +25545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="363" ht="23" customHeight="1" spans="1:20">
+    <row r="363" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A363" s="2" t="s">
         <v>1011</v>
       </c>
@@ -25596,7 +25599,7 @@
       </c>
       <c r="T363" s="2"/>
     </row>
-    <row r="364" ht="23" customHeight="1" spans="1:20">
+    <row r="364" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A364" s="2" t="s">
         <v>1013</v>
       </c>
@@ -25650,7 +25653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="365" ht="23" customHeight="1" spans="1:20">
+    <row r="365" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A365" s="2" t="s">
         <v>1015</v>
       </c>
@@ -25704,7 +25707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="366" ht="23" customHeight="1" spans="1:20">
+    <row r="366" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A366" s="2" t="s">
         <v>1017</v>
       </c>
@@ -25816,7 +25819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="368" ht="23" customHeight="1" spans="1:20">
+    <row r="368" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A368" s="2" t="s">
         <v>1022</v>
       </c>
@@ -25872,7 +25875,7 @@
       </c>
       <c r="T368" s="2"/>
     </row>
-    <row r="369" ht="23" customHeight="1" spans="1:20">
+    <row r="369" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A369" s="2" t="s">
         <v>1024</v>
       </c>
@@ -25928,7 +25931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="370" ht="23" customHeight="1" spans="1:20">
+    <row r="370" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A370" s="2" t="s">
         <v>1026</v>
       </c>
@@ -25980,7 +25983,7 @@
       <c r="S370" s="2"/>
       <c r="T370" s="2"/>
     </row>
-    <row r="371" ht="23" customHeight="1" spans="1:20">
+    <row r="371" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A371" s="2" t="s">
         <v>1028</v>
       </c>
@@ -26090,7 +26093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="373" ht="23" customHeight="1" spans="1:20">
+    <row r="373" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A373" s="2" t="s">
         <v>1033</v>
       </c>
@@ -26144,7 +26147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="374" ht="23" customHeight="1" spans="1:20">
+    <row r="374" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A374" s="2" t="s">
         <v>1034</v>
       </c>
@@ -26198,7 +26201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="375" ht="23" customHeight="1" spans="1:20">
+    <row r="375" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A375" s="2" t="s">
         <v>1036</v>
       </c>
@@ -26252,7 +26255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="376" ht="23" customHeight="1" spans="1:20">
+    <row r="376" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A376" s="2" t="s">
         <v>1039</v>
       </c>
@@ -26362,7 +26365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="378" ht="23" customHeight="1" spans="1:20">
+    <row r="378" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A378" s="2" t="s">
         <v>1041</v>
       </c>
@@ -26416,7 +26419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="379" ht="23" customHeight="1" spans="1:20">
+    <row r="379" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A379" s="2" t="s">
         <v>1044</v>
       </c>
@@ -26466,7 +26469,7 @@
       <c r="S379" s="2"/>
       <c r="T379" s="2"/>
     </row>
-    <row r="380" ht="23" customHeight="1" spans="1:20">
+    <row r="380" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A380" s="2" t="s">
         <v>1047</v>
       </c>
@@ -26522,7 +26525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="381" ht="23" customHeight="1" spans="1:20">
+    <row r="381" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A381" s="2" t="s">
         <v>1049</v>
       </c>
@@ -26634,7 +26637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="383" ht="23" customHeight="1" spans="1:20">
+    <row r="383" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A383" s="2" t="s">
         <v>1055</v>
       </c>
@@ -26688,7 +26691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="384" ht="23" customHeight="1" spans="1:20">
+    <row r="384" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A384" s="2" t="s">
         <v>1057</v>
       </c>
@@ -26738,7 +26741,7 @@
       <c r="S384" s="2"/>
       <c r="T384" s="2"/>
     </row>
-    <row r="385" ht="23" customHeight="1" spans="1:20">
+    <row r="385" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A385" s="2" t="s">
         <v>1059</v>
       </c>
@@ -26792,7 +26795,7 @@
       </c>
       <c r="T385" s="2"/>
     </row>
-    <row r="386" ht="23" customHeight="1" spans="1:20">
+    <row r="386" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A386" s="2" t="s">
         <v>1062</v>
       </c>
@@ -26904,7 +26907,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="388" ht="23" customHeight="1" spans="1:20">
+    <row r="388" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A388" s="2" t="s">
         <v>1064</v>
       </c>
@@ -26958,7 +26961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="389" ht="23" customHeight="1" spans="1:20">
+    <row r="389" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A389" s="2" t="s">
         <v>1067</v>
       </c>
@@ -27014,7 +27017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="390" ht="23" customHeight="1" spans="1:20">
+    <row r="390" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A390" s="2" t="s">
         <v>1070</v>
       </c>
@@ -27070,7 +27073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="391" ht="23" customHeight="1" spans="1:20">
+    <row r="391" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A391" s="2" t="s">
         <v>1072</v>
       </c>
@@ -27180,7 +27183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="393" ht="23" customHeight="1" spans="1:20">
+    <row r="393" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A393" s="2" t="s">
         <v>1077</v>
       </c>
@@ -27236,7 +27239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="394" ht="23" customHeight="1" spans="1:20">
+    <row r="394" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A394" s="2" t="s">
         <v>1080</v>
       </c>
@@ -27290,7 +27293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="395" ht="23" customHeight="1" spans="1:20">
+    <row r="395" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A395" s="2" t="s">
         <v>1084</v>
       </c>
@@ -27344,7 +27347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="396" ht="23" customHeight="1" spans="1:20">
+    <row r="396" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A396" s="2" t="s">
         <v>1085</v>
       </c>
@@ -27452,7 +27455,7 @@
       <c r="S397" s="2"/>
       <c r="T397" s="2"/>
     </row>
-    <row r="398" ht="23" customHeight="1" spans="1:20">
+    <row r="398" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A398" s="2" t="s">
         <v>1090</v>
       </c>
@@ -27506,7 +27509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="399" ht="23" customHeight="1" spans="1:20">
+    <row r="399" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A399" s="2" t="s">
         <v>1093</v>
       </c>
@@ -27556,7 +27559,7 @@
       <c r="S399" s="2"/>
       <c r="T399" s="2"/>
     </row>
-    <row r="400" ht="23" customHeight="1" spans="1:20">
+    <row r="400" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A400" s="2" t="s">
         <v>1095</v>
       </c>
@@ -27610,7 +27613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="401" ht="23" customHeight="1" spans="1:20">
+    <row r="401" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A401" s="2" t="s">
         <v>1098</v>
       </c>
@@ -27718,7 +27721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="403" ht="23" customHeight="1" spans="1:20">
+    <row r="403" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A403" s="2" t="s">
         <v>1104</v>
       </c>
@@ -27772,7 +27775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="404" ht="23" customHeight="1" spans="1:20">
+    <row r="404" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A404" s="2" t="s">
         <v>1105</v>
       </c>
@@ -27828,7 +27831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="405" ht="23" customHeight="1" spans="1:20">
+    <row r="405" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A405" s="2" t="s">
         <v>1107</v>
       </c>
@@ -27884,7 +27887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="406" ht="23" customHeight="1" spans="1:20">
+    <row r="406" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A406" s="2" t="s">
         <v>1109</v>
       </c>
@@ -27994,7 +27997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="408" ht="23" customHeight="1" spans="1:20">
+    <row r="408" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A408" s="2" t="s">
         <v>1114</v>
       </c>
@@ -28046,7 +28049,7 @@
       </c>
       <c r="T408" s="2"/>
     </row>
-    <row r="409" ht="23" customHeight="1" spans="1:20">
+    <row r="409" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A409" s="2" t="s">
         <v>1117</v>
       </c>
@@ -28098,7 +28101,7 @@
       </c>
       <c r="T409" s="2"/>
     </row>
-    <row r="410" ht="23" customHeight="1" spans="1:20">
+    <row r="410" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A410" s="2" t="s">
         <v>1119</v>
       </c>
@@ -28148,7 +28151,7 @@
       <c r="S410" s="2"/>
       <c r="T410" s="2"/>
     </row>
-    <row r="411" ht="23" customHeight="1" spans="1:20">
+    <row r="411" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A411" s="2" t="s">
         <v>1122</v>
       </c>
@@ -28260,7 +28263,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="413" ht="23" customHeight="1" spans="1:20">
+    <row r="413" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A413" s="2" t="s">
         <v>1127</v>
       </c>
@@ -28316,7 +28319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="414" ht="23" customHeight="1" spans="1:20">
+    <row r="414" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A414" s="2" t="s">
         <v>1130</v>
       </c>
@@ -28366,7 +28369,7 @@
       <c r="S414" s="2"/>
       <c r="T414" s="2"/>
     </row>
-    <row r="415" ht="23" customHeight="1" spans="1:20">
+    <row r="415" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A415" s="2" t="s">
         <v>1132</v>
       </c>
@@ -28420,7 +28423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="416" ht="23" customHeight="1" spans="1:20">
+    <row r="416" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A416" s="2" t="s">
         <v>1134</v>
       </c>
@@ -28530,7 +28533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="418" ht="23" customHeight="1" spans="1:20">
+    <row r="418" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A418" s="2" t="s">
         <v>1139</v>
       </c>
@@ -28586,7 +28589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="419" ht="23" customHeight="1" spans="1:20">
+    <row r="419" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A419" s="2" t="s">
         <v>1141</v>
       </c>
@@ -28642,7 +28645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="420" ht="23" customHeight="1" spans="1:20">
+    <row r="420" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A420" s="2" t="s">
         <v>1143</v>
       </c>
@@ -28698,7 +28701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="421" ht="23" customHeight="1" spans="1:20">
+    <row r="421" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A421" s="2" t="s">
         <v>1144</v>
       </c>
@@ -28808,7 +28811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="423" ht="23" customHeight="1" spans="1:20">
+    <row r="423" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A423" s="2" t="s">
         <v>1150</v>
       </c>
@@ -28864,7 +28867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="424" ht="23" customHeight="1" spans="1:20">
+    <row r="424" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A424" s="2" t="s">
         <v>1154</v>
       </c>
@@ -28920,7 +28923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="425" ht="23" customHeight="1" spans="1:20">
+    <row r="425" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A425" s="2" t="s">
         <v>1155</v>
       </c>
@@ -28976,7 +28979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="426" ht="23" customHeight="1" spans="1:20">
+    <row r="426" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A426" s="2" t="s">
         <v>1157</v>
       </c>
@@ -29086,7 +29089,7 @@
       </c>
       <c r="T427" s="2"/>
     </row>
-    <row r="428" ht="23" customHeight="1" spans="1:20">
+    <row r="428" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A428" s="2" t="s">
         <v>1162</v>
       </c>
@@ -29136,7 +29139,7 @@
       <c r="S428" s="2"/>
       <c r="T428" s="2"/>
     </row>
-    <row r="429" ht="23" customHeight="1" spans="1:20">
+    <row r="429" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A429" s="2" t="s">
         <v>1165</v>
       </c>
@@ -29190,7 +29193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="430" ht="23" customHeight="1" spans="1:20">
+    <row r="430" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A430" s="2" t="s">
         <v>1168</v>
       </c>
@@ -29244,7 +29247,7 @@
       </c>
       <c r="T430" s="2"/>
     </row>
-    <row r="431" ht="23" customHeight="1" spans="1:20">
+    <row r="431" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A431" s="2" t="s">
         <v>1171</v>
       </c>
@@ -29348,7 +29351,7 @@
       <c r="S432" s="2"/>
       <c r="T432" s="2"/>
     </row>
-    <row r="433" ht="23" customHeight="1" spans="1:20">
+    <row r="433" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A433" s="2" t="s">
         <v>1176</v>
       </c>
@@ -29402,7 +29405,7 @@
       </c>
       <c r="T433" s="2"/>
     </row>
-    <row r="434" ht="23" customHeight="1" spans="1:20">
+    <row r="434" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A434" s="2" t="s">
         <v>1178</v>
       </c>
@@ -29454,7 +29457,7 @@
       </c>
       <c r="T434" s="2"/>
     </row>
-    <row r="435" ht="23" customHeight="1" spans="1:20">
+    <row r="435" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A435" s="2" t="s">
         <v>1181</v>
       </c>
@@ -29508,7 +29511,7 @@
       </c>
       <c r="T435" s="2"/>
     </row>
-    <row r="436" ht="23" customHeight="1" spans="1:20">
+    <row r="436" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A436" s="2" t="s">
         <v>1184</v>
       </c>
@@ -29616,7 +29619,7 @@
       <c r="S437" s="2"/>
       <c r="T437" s="2"/>
     </row>
-    <row r="438" ht="23" customHeight="1" spans="1:20">
+    <row r="438" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A438" s="2" t="s">
         <v>1186</v>
       </c>
@@ -29672,7 +29675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="439" ht="23" customHeight="1" spans="1:20">
+    <row r="439" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A439" s="2" t="s">
         <v>1189</v>
       </c>
@@ -29728,7 +29731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="440" ht="23" customHeight="1" spans="1:20">
+    <row r="440" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A440" s="2" t="s">
         <v>1192</v>
       </c>
@@ -29786,7 +29789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="441" ht="23" customHeight="1" spans="1:20">
+    <row r="441" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A441" s="2" t="s">
         <v>1195</v>
       </c>
@@ -29894,7 +29897,7 @@
       <c r="S442" s="2"/>
       <c r="T442" s="2"/>
     </row>
-    <row r="443" ht="23" customHeight="1" spans="1:20">
+    <row r="443" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A443" s="2" t="s">
         <v>1200</v>
       </c>
@@ -29948,7 +29951,7 @@
       </c>
       <c r="T443" s="2"/>
     </row>
-    <row r="444" ht="23" customHeight="1" spans="1:20">
+    <row r="444" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A444" s="2" t="s">
         <v>1202</v>
       </c>
@@ -29998,7 +30001,7 @@
       <c r="S444" s="2"/>
       <c r="T444" s="2"/>
     </row>
-    <row r="445" ht="23" customHeight="1" spans="1:20">
+    <row r="445" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A445" s="2" t="s">
         <v>1204</v>
       </c>
@@ -30054,7 +30057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="446" ht="23" customHeight="1" spans="1:20">
+    <row r="446" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A446" s="2" t="s">
         <v>1206</v>
       </c>
@@ -30110,7 +30113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="447" ht="23" customHeight="1" spans="1:20">
+    <row r="447" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A447" s="2" t="s">
         <v>1208</v>
       </c>
@@ -30216,7 +30219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="449" ht="23" customHeight="1" spans="1:20">
+    <row r="449" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A449" s="2" t="s">
         <v>1212</v>
       </c>
@@ -30266,7 +30269,7 @@
       <c r="S449" s="2"/>
       <c r="T449" s="2"/>
     </row>
-    <row r="450" ht="23" customHeight="1" spans="1:20">
+    <row r="450" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A450" s="2" t="s">
         <v>1215</v>
       </c>
@@ -30318,7 +30321,7 @@
       <c r="S450" s="2"/>
       <c r="T450" s="2"/>
     </row>
-    <row r="451" ht="23" customHeight="1" spans="1:20">
+    <row r="451" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A451" s="2" t="s">
         <v>1217</v>
       </c>
@@ -30424,7 +30427,7 @@
       <c r="S452" s="2"/>
       <c r="T452" s="2"/>
     </row>
-    <row r="453" ht="23" customHeight="1" spans="1:20">
+    <row r="453" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A453" s="2" t="s">
         <v>1221</v>
       </c>
@@ -30476,7 +30479,7 @@
       <c r="S453" s="2"/>
       <c r="T453" s="2"/>
     </row>
-    <row r="454" ht="23" customHeight="1" spans="1:20">
+    <row r="454" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A454" s="2" t="s">
         <v>1223</v>
       </c>
@@ -30532,7 +30535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="455" ht="23" customHeight="1" spans="1:20">
+    <row r="455" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A455" s="2" t="s">
         <v>1224</v>
       </c>
@@ -30588,7 +30591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="456" ht="23" customHeight="1" spans="1:20">
+    <row r="456" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A456" s="2" t="s">
         <v>1226</v>
       </c>
@@ -30694,7 +30697,7 @@
       <c r="S457" s="2"/>
       <c r="T457" s="2"/>
     </row>
-    <row r="458" ht="23" customHeight="1" spans="1:20">
+    <row r="458" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A458" s="2" t="s">
         <v>1231</v>
       </c>
@@ -30750,7 +30753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="459" ht="23" customHeight="1" spans="1:20">
+    <row r="459" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A459" s="2" t="s">
         <v>1234</v>
       </c>
@@ -30806,7 +30809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="460" ht="23" customHeight="1" spans="1:20">
+    <row r="460" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A460" s="2" t="s">
         <v>1236</v>
       </c>
@@ -30862,7 +30865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="461" ht="23" customHeight="1" spans="1:20">
+    <row r="461" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A461" s="2" t="s">
         <v>1239</v>
       </c>
@@ -30964,7 +30967,7 @@
       <c r="S462" s="2"/>
       <c r="T462" s="2"/>
     </row>
-    <row r="463" ht="23" customHeight="1" spans="1:20">
+    <row r="463" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A463" s="2" t="s">
         <v>1243</v>
       </c>
@@ -31018,7 +31021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="464" ht="23" customHeight="1" spans="1:20">
+    <row r="464" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A464" s="2" t="s">
         <v>1245</v>
       </c>
@@ -31072,7 +31075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="465" ht="23" customHeight="1" spans="1:20">
+    <row r="465" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A465" s="2" t="s">
         <v>1247</v>
       </c>
@@ -31124,7 +31127,7 @@
       <c r="S465" s="2"/>
       <c r="T465" s="2"/>
     </row>
-    <row r="466" ht="23" customHeight="1" spans="1:20">
+    <row r="466" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A466" s="2" t="s">
         <v>1250</v>
       </c>
@@ -31180,7 +31183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="467" ht="23" customHeight="1" spans="1:20">
+    <row r="467" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A467" s="2" t="s">
         <v>1252</v>
       </c>
@@ -31236,7 +31239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="468" ht="23" customHeight="1" spans="1:20">
+    <row r="468" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A468" s="2" t="s">
         <v>1255</v>
       </c>
@@ -31288,7 +31291,7 @@
       <c r="S468" s="2"/>
       <c r="T468" s="2"/>
     </row>
-    <row r="469" ht="23" customHeight="1" spans="1:20">
+    <row r="469" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A469" s="2" t="s">
         <v>1257</v>
       </c>
@@ -31346,7 +31349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="470" ht="23" customHeight="1" spans="1:20">
+    <row r="470" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A470" s="2" t="s">
         <v>1260</v>
       </c>
@@ -31400,7 +31403,7 @@
       <c r="S470" s="2"/>
       <c r="T470" s="2"/>
     </row>
-    <row r="471" ht="23" customHeight="1" spans="1:20">
+    <row r="471" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A471" s="2" t="s">
         <v>1262</v>
       </c>
@@ -31506,7 +31509,7 @@
       <c r="S472" s="2"/>
       <c r="T472" s="2"/>
     </row>
-    <row r="473" ht="23" customHeight="1" spans="1:20">
+    <row r="473" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A473" s="2" t="s">
         <v>1267</v>
       </c>
@@ -31560,7 +31563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="474" ht="23" customHeight="1" spans="1:20">
+    <row r="474" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A474" s="2" t="s">
         <v>1270</v>
       </c>
@@ -31616,7 +31619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="475" ht="23" customHeight="1" spans="1:20">
+    <row r="475" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A475" s="2" t="s">
         <v>1272</v>
       </c>
@@ -31674,7 +31677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="476" ht="23" customHeight="1" spans="1:20">
+    <row r="476" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A476" s="2" t="s">
         <v>1275</v>
       </c>
@@ -31776,7 +31779,7 @@
       <c r="S477" s="2"/>
       <c r="T477" s="2"/>
     </row>
-    <row r="478" ht="23" customHeight="1" spans="1:20">
+    <row r="478" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A478" s="2" t="s">
         <v>1280</v>
       </c>
@@ -31830,7 +31833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="479" ht="23" customHeight="1" spans="1:20">
+    <row r="479" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A479" s="2" t="s">
         <v>1283</v>
       </c>
@@ -31882,7 +31885,7 @@
       </c>
       <c r="T479" s="2"/>
     </row>
-    <row r="480" ht="23" customHeight="1" spans="1:20">
+    <row r="480" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A480" s="2" t="s">
         <v>1286</v>
       </c>
@@ -31932,7 +31935,7 @@
       <c r="S480" s="2"/>
       <c r="T480" s="2"/>
     </row>
-    <row r="481" ht="23" customHeight="1" spans="1:20">
+    <row r="481" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A481" s="2" t="s">
         <v>1289</v>
       </c>
@@ -32042,7 +32045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="483" ht="23" customHeight="1" spans="1:20">
+    <row r="483" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A483" s="2" t="s">
         <v>1293</v>
       </c>
@@ -32094,7 +32097,7 @@
       </c>
       <c r="T483" s="2"/>
     </row>
-    <row r="484" ht="23" customHeight="1" spans="1:20">
+    <row r="484" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A484" s="2" t="s">
         <v>1295</v>
       </c>
@@ -32148,7 +32151,7 @@
       <c r="S484" s="2"/>
       <c r="T484" s="2"/>
     </row>
-    <row r="485" ht="23" customHeight="1" spans="1:20">
+    <row r="485" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A485" s="2" t="s">
         <v>1296</v>
       </c>
@@ -32202,7 +32205,7 @@
       </c>
       <c r="T485" s="2"/>
     </row>
-    <row r="486" ht="23" customHeight="1" spans="1:20">
+    <row r="486" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A486" s="2" t="s">
         <v>1298</v>
       </c>
@@ -32254,7 +32257,7 @@
       <c r="S486" s="2"/>
       <c r="T486" s="2"/>
     </row>
-    <row r="487" ht="23" customHeight="1" spans="1:20">
+    <row r="487" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A487" s="2" t="s">
         <v>1300</v>
       </c>
@@ -32364,7 +32367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="489" ht="23" customHeight="1" spans="1:20">
+    <row r="489" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A489" s="2" t="s">
         <v>1305</v>
       </c>
@@ -32418,7 +32421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="490" ht="23" customHeight="1" spans="1:20">
+    <row r="490" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A490" s="2" t="s">
         <v>1307</v>
       </c>
@@ -32470,7 +32473,7 @@
       <c r="S490" s="2"/>
       <c r="T490" s="2"/>
     </row>
-    <row r="491" ht="23" customHeight="1" spans="1:20">
+    <row r="491" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A491" s="2" t="s">
         <v>1311</v>
       </c>
@@ -32524,7 +32527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="492" ht="23" customHeight="1" spans="1:20">
+    <row r="492" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A492" s="2" t="s">
         <v>1313</v>
       </c>
@@ -32632,7 +32635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="494" ht="23" customHeight="1" spans="1:20">
+    <row r="494" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A494" s="2" t="s">
         <v>1318</v>
       </c>
@@ -32682,7 +32685,7 @@
       <c r="S494" s="2"/>
       <c r="T494" s="2"/>
     </row>
-    <row r="495" ht="23" customHeight="1" spans="1:20">
+    <row r="495" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A495" s="2" t="s">
         <v>1321</v>
       </c>
@@ -32738,7 +32741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="496" ht="23" customHeight="1" spans="1:20">
+    <row r="496" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A496" s="2" t="s">
         <v>1323</v>
       </c>
@@ -32794,7 +32797,7 @@
       </c>
       <c r="T496" s="2"/>
     </row>
-    <row r="497" ht="23" customHeight="1" spans="1:20">
+    <row r="497" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A497" s="2" t="s">
         <v>1325</v>
       </c>
@@ -32904,7 +32907,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="499" ht="23" customHeight="1" spans="1:20">
+    <row r="499" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A499" s="2" t="s">
         <v>1329</v>
       </c>
@@ -32958,7 +32961,7 @@
       </c>
       <c r="T499" s="2"/>
     </row>
-    <row r="500" ht="23" customHeight="1" spans="1:20">
+    <row r="500" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A500" s="2" t="s">
         <v>1332</v>
       </c>
@@ -33014,7 +33017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="501" ht="23" customHeight="1" spans="1:20">
+    <row r="501" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A501" s="2" t="s">
         <v>1334</v>
       </c>
@@ -33068,7 +33071,7 @@
       </c>
       <c r="T501" s="2"/>
     </row>
-    <row r="502" ht="23" customHeight="1" spans="1:20">
+    <row r="502" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A502" s="2" t="s">
         <v>1336</v>
       </c>
@@ -33178,7 +33181,7 @@
       </c>
       <c r="T503" s="2"/>
     </row>
-    <row r="504" ht="23" customHeight="1" spans="1:20">
+    <row r="504" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A504" s="2" t="s">
         <v>1340</v>
       </c>
@@ -33232,7 +33235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="505" ht="23" customHeight="1" spans="1:20">
+    <row r="505" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A505" s="2" t="s">
         <v>1342</v>
       </c>
@@ -33288,7 +33291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="506" ht="23" customHeight="1" spans="1:20">
+    <row r="506" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A506" s="2" t="s">
         <v>1344</v>
       </c>
@@ -33342,7 +33345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="507" ht="23" customHeight="1" spans="1:20">
+    <row r="507" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A507" s="2" t="s">
         <v>1346</v>
       </c>
@@ -33452,7 +33455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="509" ht="23" customHeight="1" spans="1:20">
+    <row r="509" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A509" s="2" t="s">
         <v>1351</v>
       </c>
@@ -33508,7 +33511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="510" ht="23" customHeight="1" spans="1:20">
+    <row r="510" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A510" s="2" t="s">
         <v>1352</v>
       </c>
@@ -33564,7 +33567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="511" ht="23" customHeight="1" spans="1:20">
+    <row r="511" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A511" s="2" t="s">
         <v>1354</v>
       </c>
@@ -33618,7 +33621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="512" ht="23" customHeight="1" spans="1:20">
+    <row r="512" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A512" s="2" t="s">
         <v>1356</v>
       </c>
@@ -33726,7 +33729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="514" ht="23" customHeight="1" spans="1:20">
+    <row r="514" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A514" s="2" t="s">
         <v>1360</v>
       </c>
@@ -33780,7 +33783,7 @@
       </c>
       <c r="T514" s="2"/>
     </row>
-    <row r="515" ht="23" customHeight="1" spans="1:20">
+    <row r="515" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A515" s="2" t="s">
         <v>1363</v>
       </c>
@@ -33832,7 +33835,7 @@
       <c r="S515" s="2"/>
       <c r="T515" s="2"/>
     </row>
-    <row r="516" ht="23" customHeight="1" spans="1:20">
+    <row r="516" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A516" s="2" t="s">
         <v>1366</v>
       </c>
@@ -33886,7 +33889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="517" ht="23" customHeight="1" spans="1:20">
+    <row r="517" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A517" s="2" t="s">
         <v>1368</v>
       </c>
@@ -33998,7 +34001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="519" ht="23" customHeight="1" spans="1:20">
+    <row r="519" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A519" s="2" t="s">
         <v>1373</v>
       </c>
@@ -34054,7 +34057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="520" ht="23" customHeight="1" spans="1:20">
+    <row r="520" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A520" s="2" t="s">
         <v>1374</v>
       </c>
@@ -34104,7 +34107,7 @@
       <c r="S520" s="2"/>
       <c r="T520" s="2"/>
     </row>
-    <row r="521" ht="23" customHeight="1" spans="1:20">
+    <row r="521" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A521" s="2" t="s">
         <v>1376</v>
       </c>
@@ -34158,7 +34161,7 @@
       </c>
       <c r="T521" s="2"/>
     </row>
-    <row r="522" ht="23" customHeight="1" spans="1:20">
+    <row r="522" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A522" s="2" t="s">
         <v>1377</v>
       </c>
@@ -34268,7 +34271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="524" ht="23" customHeight="1" spans="1:20">
+    <row r="524" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A524" s="2" t="s">
         <v>1381</v>
       </c>
@@ -34322,7 +34325,7 @@
       </c>
       <c r="T524" s="2"/>
     </row>
-    <row r="525" ht="23" customHeight="1" spans="1:20">
+    <row r="525" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A525" s="2" t="s">
         <v>1384</v>
       </c>
@@ -34376,7 +34379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="526" ht="23" customHeight="1" spans="1:20">
+    <row r="526" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A526" s="2" t="s">
         <v>1386</v>
       </c>
@@ -34432,7 +34435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="527" ht="23" customHeight="1" spans="1:20">
+    <row r="527" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A527" s="2" t="s">
         <v>1387</v>
       </c>
@@ -34540,7 +34543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="529" ht="23" customHeight="1" spans="1:20">
+    <row r="529" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A529" s="2" t="s">
         <v>1391</v>
       </c>
@@ -34596,7 +34599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="530" ht="23" customHeight="1" spans="1:20">
+    <row r="530" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A530" s="2" t="s">
         <v>1394</v>
       </c>
@@ -34650,7 +34653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="531" ht="23" customHeight="1" spans="1:20">
+    <row r="531" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A531" s="2" t="s">
         <v>1396</v>
       </c>
@@ -34706,7 +34709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="532" ht="23" customHeight="1" spans="1:20">
+    <row r="532" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A532" s="2" t="s">
         <v>1398</v>
       </c>
@@ -34814,7 +34817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="534" ht="23" customHeight="1" spans="1:20">
+    <row r="534" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A534" s="2" t="s">
         <v>1402</v>
       </c>
@@ -34870,7 +34873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="535" ht="23" customHeight="1" spans="1:20">
+    <row r="535" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A535" s="2" t="s">
         <v>1404</v>
       </c>
@@ -34924,7 +34927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="536" ht="23" customHeight="1" spans="1:20">
+    <row r="536" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A536" s="2" t="s">
         <v>1406</v>
       </c>
@@ -34976,7 +34979,7 @@
       <c r="S536" s="2"/>
       <c r="T536" s="2"/>
     </row>
-    <row r="537" ht="23" customHeight="1" spans="1:20">
+    <row r="537" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A537" s="2" t="s">
         <v>1409</v>
       </c>
@@ -35086,7 +35089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="539" ht="23" customHeight="1" spans="1:20">
+    <row r="539" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A539" s="2" t="s">
         <v>1414</v>
       </c>
@@ -35140,7 +35143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="540" ht="23" customHeight="1" spans="1:20">
+    <row r="540" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A540" s="2" t="s">
         <v>1417</v>
       </c>
@@ -35192,7 +35195,7 @@
       <c r="S540" s="2"/>
       <c r="T540" s="2"/>
     </row>
-    <row r="541" ht="23" customHeight="1" spans="1:20">
+    <row r="541" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A541" s="2" t="s">
         <v>1420</v>
       </c>
@@ -35242,7 +35245,7 @@
       <c r="S541" s="2"/>
       <c r="T541" s="2"/>
     </row>
-    <row r="542" ht="23" customHeight="1" spans="1:20">
+    <row r="542" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A542" s="2" t="s">
         <v>1423</v>
       </c>
@@ -35348,7 +35351,7 @@
       <c r="S543" s="2"/>
       <c r="T543" s="2"/>
     </row>
-    <row r="544" ht="23" customHeight="1" spans="1:20">
+    <row r="544" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A544" s="2" t="s">
         <v>1428</v>
       </c>
@@ -35406,7 +35409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="545" ht="23" customHeight="1" spans="1:20">
+    <row r="545" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A545" s="2" t="s">
         <v>1431</v>
       </c>
@@ -35458,7 +35461,7 @@
       <c r="S545" s="2"/>
       <c r="T545" s="2"/>
     </row>
-    <row r="546" ht="23" customHeight="1" spans="1:20">
+    <row r="546" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A546" s="2" t="s">
         <v>1433</v>
       </c>
@@ -35514,7 +35517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="547" ht="23" customHeight="1" spans="1:20">
+    <row r="547" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A547" s="2" t="s">
         <v>1435</v>
       </c>
@@ -35624,7 +35627,7 @@
       </c>
       <c r="T548" s="2"/>
     </row>
-    <row r="549" ht="23" customHeight="1" spans="1:20">
+    <row r="549" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A549" s="2" t="s">
         <v>1439</v>
       </c>
@@ -35680,7 +35683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="550" ht="23" customHeight="1" spans="1:20">
+    <row r="550" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A550" s="2" t="s">
         <v>1442</v>
       </c>
@@ -35736,7 +35739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="551" ht="23" customHeight="1" spans="1:20">
+    <row r="551" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A551" s="2" t="s">
         <v>1443</v>
       </c>
@@ -35790,7 +35793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="552" ht="23" customHeight="1" spans="1:20">
+    <row r="552" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A552" s="2" t="s">
         <v>1444</v>
       </c>
@@ -35900,7 +35903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="554" ht="23" customHeight="1" spans="1:20">
+    <row r="554" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A554" s="2" t="s">
         <v>1450</v>
       </c>
@@ -35952,7 +35955,7 @@
       <c r="S554" s="2"/>
       <c r="T554" s="2"/>
     </row>
-    <row r="555" ht="23" customHeight="1" spans="1:20">
+    <row r="555" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A555" s="2" t="s">
         <v>1452</v>
       </c>
@@ -36008,7 +36011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="556" ht="23" customHeight="1" spans="1:20">
+    <row r="556" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A556" s="2" t="s">
         <v>1454</v>
       </c>
@@ -36062,7 +36065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="557" ht="23" customHeight="1" spans="1:20">
+    <row r="557" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A557" s="2" t="s">
         <v>1455</v>
       </c>
@@ -36170,7 +36173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="559" ht="23" customHeight="1" spans="1:20">
+    <row r="559" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A559" s="2" t="s">
         <v>1461</v>
       </c>
@@ -36224,7 +36227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="560" ht="23" customHeight="1" spans="1:20">
+    <row r="560" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A560" s="2" t="s">
         <v>1462</v>
       </c>
@@ -36280,7 +36283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="561" ht="23" customHeight="1" spans="1:20">
+    <row r="561" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A561" s="2" t="s">
         <v>1464</v>
       </c>
@@ -36334,7 +36337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="562" ht="23" customHeight="1" spans="1:20">
+    <row r="562" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A562" s="2" t="s">
         <v>1466</v>
       </c>
@@ -36446,7 +36449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="564" ht="23" customHeight="1" spans="1:20">
+    <row r="564" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A564" s="2" t="s">
         <v>1470</v>
       </c>
@@ -36502,7 +36505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="565" ht="23" customHeight="1" spans="1:20">
+    <row r="565" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A565" s="2" t="s">
         <v>1471</v>
       </c>
@@ -36556,7 +36559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="566" ht="23" customHeight="1" spans="1:20">
+    <row r="566" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A566" s="2" t="s">
         <v>1473</v>
       </c>
@@ -36608,7 +36611,7 @@
       </c>
       <c r="T566" s="2"/>
     </row>
-    <row r="567" ht="23" customHeight="1" spans="1:20">
+    <row r="567" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A567" s="2" t="s">
         <v>1475</v>
       </c>
@@ -36720,7 +36723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="569" ht="23" customHeight="1" spans="1:20">
+    <row r="569" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A569" s="2" t="s">
         <v>1480</v>
       </c>
@@ -36772,7 +36775,7 @@
       </c>
       <c r="T569" s="2"/>
     </row>
-    <row r="570" ht="23" customHeight="1" spans="1:20">
+    <row r="570" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A570" s="2" t="s">
         <v>1482</v>
       </c>
@@ -36826,7 +36829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="571" ht="23" customHeight="1" spans="1:20">
+    <row r="571" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A571" s="2" t="s">
         <v>1484</v>
       </c>
@@ -36880,7 +36883,7 @@
       </c>
       <c r="T571" s="2"/>
     </row>
-    <row r="572" ht="23" customHeight="1" spans="1:20">
+    <row r="572" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A572" s="2" t="s">
         <v>1487</v>
       </c>
@@ -36990,7 +36993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="574" ht="23" customHeight="1" spans="1:20">
+    <row r="574" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A574" s="2" t="s">
         <v>1492</v>
       </c>
@@ -37044,7 +37047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="575" ht="23" customHeight="1" spans="1:20">
+    <row r="575" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A575" s="2" t="s">
         <v>1494</v>
       </c>
@@ -37100,7 +37103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="576" ht="23" customHeight="1" spans="1:20">
+    <row r="576" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A576" s="2" t="s">
         <v>1496</v>
       </c>
@@ -37154,7 +37157,7 @@
       </c>
       <c r="T576" s="2"/>
     </row>
-    <row r="577" ht="23" customHeight="1" spans="1:20">
+    <row r="577" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A577" s="2" t="s">
         <v>1499</v>
       </c>
@@ -37262,7 +37265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="579" ht="23" customHeight="1" spans="1:20">
+    <row r="579" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A579" s="2" t="s">
         <v>1502</v>
       </c>
@@ -37316,7 +37319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="580" ht="23" customHeight="1" spans="1:20">
+    <row r="580" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A580" s="2" t="s">
         <v>1505</v>
       </c>
@@ -37370,7 +37373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="581" ht="23" customHeight="1" spans="1:20">
+    <row r="581" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A581" s="2" t="s">
         <v>1508</v>
       </c>
@@ -37424,7 +37427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="582" ht="23" customHeight="1" spans="1:20">
+    <row r="582" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A582" s="2" t="s">
         <v>1510</v>
       </c>
@@ -37532,7 +37535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="584" ht="23" customHeight="1" spans="1:20">
+    <row r="584" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A584" s="2" t="s">
         <v>1514</v>
       </c>
@@ -37590,7 +37593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="585" ht="23" customHeight="1" spans="1:20">
+    <row r="585" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A585" s="2" t="s">
         <v>1516</v>
       </c>
@@ -37644,7 +37647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="586" ht="23" customHeight="1" spans="1:20">
+    <row r="586" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A586" s="2" t="s">
         <v>1518</v>
       </c>
@@ -37698,7 +37701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="587" ht="23" customHeight="1" spans="1:20">
+    <row r="587" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A587" s="2" t="s">
         <v>1521</v>
       </c>
@@ -37806,7 +37809,7 @@
       <c r="S588" s="2"/>
       <c r="T588" s="2"/>
     </row>
-    <row r="589" ht="23" customHeight="1" spans="1:20">
+    <row r="589" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A589" s="2" t="s">
         <v>1525</v>
       </c>
@@ -37858,7 +37861,7 @@
       <c r="S589" s="2"/>
       <c r="T589" s="2"/>
     </row>
-    <row r="590" ht="23" customHeight="1" spans="1:20">
+    <row r="590" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A590" s="2" t="s">
         <v>1527</v>
       </c>
@@ -37912,7 +37915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="591" ht="23" customHeight="1" spans="1:20">
+    <row r="591" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A591" s="2" t="s">
         <v>1530</v>
       </c>
@@ -37968,7 +37971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="592" ht="23" customHeight="1" spans="1:20">
+    <row r="592" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A592" s="2" t="s">
         <v>1532</v>
       </c>
@@ -38078,7 +38081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="594" ht="23" customHeight="1" spans="1:20">
+    <row r="594" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A594" s="2" t="s">
         <v>1535</v>
       </c>
@@ -38130,7 +38133,7 @@
       </c>
       <c r="T594" s="2"/>
     </row>
-    <row r="595" ht="23" customHeight="1" spans="1:20">
+    <row r="595" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A595" s="2" t="s">
         <v>1537</v>
       </c>
@@ -38182,7 +38185,7 @@
       <c r="S595" s="2"/>
       <c r="T595" s="2"/>
     </row>
-    <row r="596" ht="23" customHeight="1" spans="1:20">
+    <row r="596" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A596" s="2" t="s">
         <v>1538</v>
       </c>
@@ -38236,7 +38239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="597" ht="23" customHeight="1" spans="1:20">
+    <row r="597" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A597" s="2" t="s">
         <v>1542</v>
       </c>
@@ -38344,7 +38347,7 @@
       <c r="S598" s="2"/>
       <c r="T598" s="2"/>
     </row>
-    <row r="599" ht="23" customHeight="1" spans="1:20">
+    <row r="599" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A599" s="2" t="s">
         <v>1546</v>
       </c>
@@ -38400,7 +38403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="600" ht="23" customHeight="1" spans="1:20">
+    <row r="600" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A600" s="2" t="s">
         <v>1548</v>
       </c>
@@ -38454,7 +38457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="601" ht="23" customHeight="1" spans="1:20">
+    <row r="601" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A601" s="2" t="s">
         <v>1550</v>
       </c>
@@ -38506,7 +38509,7 @@
       <c r="S601" s="2"/>
       <c r="T601" s="2"/>
     </row>
-    <row r="602" ht="23" customHeight="1" spans="1:20">
+    <row r="602" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A602" s="2" t="s">
         <v>1553</v>
       </c>
@@ -38610,7 +38613,7 @@
       </c>
       <c r="T603" s="2"/>
     </row>
-    <row r="604" ht="23" customHeight="1" spans="1:20">
+    <row r="604" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A604" s="2" t="s">
         <v>1557</v>
       </c>
@@ -38666,7 +38669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="605" ht="23" customHeight="1" spans="1:20">
+    <row r="605" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A605" s="2" t="s">
         <v>1558</v>
       </c>
@@ -38722,7 +38725,7 @@
       </c>
       <c r="T605" s="2"/>
     </row>
-    <row r="606" ht="23" customHeight="1" spans="1:20">
+    <row r="606" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A606" s="2" t="s">
         <v>1560</v>
       </c>
@@ -38778,7 +38781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="607" ht="23" customHeight="1" spans="1:20">
+    <row r="607" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A607" s="2" t="s">
         <v>1563</v>
       </c>
@@ -38890,7 +38893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="609" ht="23" customHeight="1" spans="1:20">
+    <row r="609" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A609" s="2" t="s">
         <v>1567</v>
       </c>
@@ -38946,7 +38949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="610" ht="23" customHeight="1" spans="1:20">
+    <row r="610" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A610" s="2" t="s">
         <v>1569</v>
       </c>
@@ -39000,7 +39003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="611" ht="23" customHeight="1" spans="1:20">
+    <row r="611" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A611" s="2" t="s">
         <v>1570</v>
       </c>
@@ -39054,7 +39057,7 @@
       </c>
       <c r="T611" s="2"/>
     </row>
-    <row r="612" ht="23" customHeight="1" spans="1:20">
+    <row r="612" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A612" s="2" t="s">
         <v>1571</v>
       </c>
@@ -39160,7 +39163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="614" ht="23" customHeight="1" spans="1:20">
+    <row r="614" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A614" s="2" t="s">
         <v>1576</v>
       </c>
@@ -39212,7 +39215,7 @@
       </c>
       <c r="T614" s="2"/>
     </row>
-    <row r="615" ht="23" customHeight="1" spans="1:20">
+    <row r="615" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A615" s="2" t="s">
         <v>1579</v>
       </c>
@@ -39268,7 +39271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="616" ht="23" customHeight="1" spans="1:20">
+    <row r="616" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A616" s="2" t="s">
         <v>1581</v>
       </c>
@@ -39324,7 +39327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="617" ht="23" customHeight="1" spans="1:20">
+    <row r="617" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A617" s="2" t="s">
         <v>1582</v>
       </c>
@@ -39432,7 +39435,7 @@
       </c>
       <c r="T618" s="2"/>
     </row>
-    <row r="619" ht="23" customHeight="1" spans="1:20">
+    <row r="619" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A619" s="2" t="s">
         <v>1587</v>
       </c>
@@ -39484,7 +39487,7 @@
       </c>
       <c r="T619" s="2"/>
     </row>
-    <row r="620" ht="23" customHeight="1" spans="1:20">
+    <row r="620" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A620" s="2" t="s">
         <v>1590</v>
       </c>
@@ -39534,7 +39537,7 @@
       <c r="S620" s="2"/>
       <c r="T620" s="2"/>
     </row>
-    <row r="621" ht="23" customHeight="1" spans="1:20">
+    <row r="621" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A621" s="2" t="s">
         <v>1592</v>
       </c>
@@ -39584,7 +39587,7 @@
       <c r="S621" s="2"/>
       <c r="T621" s="2"/>
     </row>
-    <row r="622" ht="23" customHeight="1" spans="1:20">
+    <row r="622" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A622" s="2" t="s">
         <v>1595</v>
       </c>
@@ -39694,7 +39697,7 @@
       </c>
       <c r="T623" s="2"/>
     </row>
-    <row r="624" ht="23" customHeight="1" spans="1:20">
+    <row r="624" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A624" s="2" t="s">
         <v>1599</v>
       </c>
@@ -39748,7 +39751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="625" ht="23" customHeight="1" spans="1:20">
+    <row r="625" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A625" s="2" t="s">
         <v>1601</v>
       </c>
@@ -39800,7 +39803,7 @@
       <c r="S625" s="2"/>
       <c r="T625" s="2"/>
     </row>
-    <row r="626" ht="23" customHeight="1" spans="1:20">
+    <row r="626" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A626" s="2" t="s">
         <v>1604</v>
       </c>
@@ -39856,7 +39859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="627" ht="23" customHeight="1" spans="1:20">
+    <row r="627" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A627" s="2" t="s">
         <v>1607</v>
       </c>
@@ -39966,7 +39969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="629" ht="23" customHeight="1" spans="1:20">
+    <row r="629" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A629" s="2" t="s">
         <v>1612</v>
       </c>
@@ -40018,7 +40021,7 @@
       </c>
       <c r="T629" s="2"/>
     </row>
-    <row r="630" ht="23" customHeight="1" spans="1:20">
+    <row r="630" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A630" s="2" t="s">
         <v>1614</v>
       </c>
@@ -40076,7 +40079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="631" ht="23" customHeight="1" spans="1:20">
+    <row r="631" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A631" s="2" t="s">
         <v>1616</v>
       </c>
@@ -40128,7 +40131,7 @@
       <c r="S631" s="2"/>
       <c r="T631" s="2"/>
     </row>
-    <row r="632" ht="23" customHeight="1" spans="1:20">
+    <row r="632" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A632" s="2" t="s">
         <v>1618</v>
       </c>
@@ -40240,7 +40243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="634" ht="23" customHeight="1" spans="1:20">
+    <row r="634" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A634" s="2" t="s">
         <v>1622</v>
       </c>
@@ -40296,7 +40299,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="635" ht="23" customHeight="1" spans="1:20">
+    <row r="635" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A635" s="2" t="s">
         <v>1624</v>
       </c>
@@ -40350,7 +40353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="636" ht="23" customHeight="1" spans="1:20">
+    <row r="636" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A636" s="2" t="s">
         <v>1626</v>
       </c>
@@ -40406,7 +40409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="637" ht="23" customHeight="1" spans="1:20">
+    <row r="637" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A637" s="2" t="s">
         <v>1628</v>
       </c>
@@ -40518,7 +40521,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="639" ht="23" customHeight="1" spans="1:20">
+    <row r="639" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A639" s="2" t="s">
         <v>1631</v>
       </c>
@@ -40574,7 +40577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="640" ht="23" customHeight="1" spans="1:20">
+    <row r="640" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A640" s="2" t="s">
         <v>1634</v>
       </c>
@@ -40626,7 +40629,7 @@
       <c r="S640" s="2"/>
       <c r="T640" s="2"/>
     </row>
-    <row r="641" ht="23" customHeight="1" spans="1:20">
+    <row r="641" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A641" s="2" t="s">
         <v>1636</v>
       </c>
@@ -40682,7 +40685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="642" ht="23" customHeight="1" spans="1:20">
+    <row r="642" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A642" s="2" t="s">
         <v>1637</v>
       </c>
@@ -40790,7 +40793,7 @@
       </c>
       <c r="T643" s="2"/>
     </row>
-    <row r="644" ht="23" customHeight="1" spans="1:20">
+    <row r="644" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A644" s="2" t="s">
         <v>1642</v>
       </c>
@@ -40846,7 +40849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="645" ht="23" customHeight="1" spans="1:20">
+    <row r="645" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A645" s="2" t="s">
         <v>1644</v>
       </c>
@@ -40896,7 +40899,7 @@
       <c r="S645" s="2"/>
       <c r="T645" s="2"/>
     </row>
-    <row r="646" ht="23" customHeight="1" spans="1:20">
+    <row r="646" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A646" s="2" t="s">
         <v>1646</v>
       </c>
@@ -40948,7 +40951,7 @@
       <c r="S646" s="2"/>
       <c r="T646" s="2"/>
     </row>
-    <row r="647" ht="23" customHeight="1" spans="1:20">
+    <row r="647" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A647" s="2" t="s">
         <v>1648</v>
       </c>
@@ -41056,7 +41059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="649" ht="23" customHeight="1" spans="1:20">
+    <row r="649" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A649" s="2" t="s">
         <v>1653</v>
       </c>
@@ -41112,7 +41115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="650" ht="23" customHeight="1" spans="1:20">
+    <row r="650" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A650" s="2" t="s">
         <v>1655</v>
       </c>
@@ -41164,7 +41167,7 @@
       <c r="S650" s="2"/>
       <c r="T650" s="2"/>
     </row>
-    <row r="651" ht="23" customHeight="1" spans="1:20">
+    <row r="651" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A651" s="2" t="s">
         <v>1657</v>
       </c>
@@ -41218,7 +41221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="652" ht="23" customHeight="1" spans="1:20">
+    <row r="652" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A652" s="2" t="s">
         <v>1659</v>
       </c>
@@ -41324,7 +41327,7 @@
       <c r="S653" s="2"/>
       <c r="T653" s="2"/>
     </row>
-    <row r="654" ht="23" customHeight="1" spans="1:20">
+    <row r="654" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A654" s="2" t="s">
         <v>1665</v>
       </c>
@@ -41380,7 +41383,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="655" ht="23" customHeight="1" spans="1:20">
+    <row r="655" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A655" s="2" t="s">
         <v>1666</v>
       </c>
@@ -41434,7 +41437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="656" ht="23" customHeight="1" spans="1:20">
+    <row r="656" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A656" s="2" t="s">
         <v>1667</v>
       </c>
@@ -41490,7 +41493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="657" ht="23" customHeight="1" spans="1:20">
+    <row r="657" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A657" s="2" t="s">
         <v>1670</v>
       </c>
@@ -41596,7 +41599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="659" ht="23" customHeight="1" spans="1:20">
+    <row r="659" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A659" s="2" t="s">
         <v>1676</v>
       </c>
@@ -41650,7 +41653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="660" ht="23" customHeight="1" spans="1:20">
+    <row r="660" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A660" s="2" t="s">
         <v>1678</v>
       </c>
@@ -41704,7 +41707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="661" ht="23" customHeight="1" spans="1:20">
+    <row r="661" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A661" s="2" t="s">
         <v>1681</v>
       </c>
@@ -41758,7 +41761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="662" ht="23" customHeight="1" spans="1:20">
+    <row r="662" ht="23" hidden="1" customHeight="1" spans="1:20">
       <c r="A662" s="2" t="s">
         <v>1683</v>
       </c>
@@ -41815,6 +41818,14 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:T662" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="carolina.gutierrez"/>
+      </filters>
+    </filterColumn>
+    <extLst/>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="F381" r:id="rId1" display="https://partners-manager.rappi.com/hunter-tools/commercial-processes/155ac9c2-6948-4d7e-a06c-d5f84da9a556" tooltip="https://partners-manager.rappi.com/hunter-tools/commercial-processes/155ac9c2-6948-4d7e-a06c-d5f84da9a556"/>
   </hyperlinks>

</xml_diff>